<commit_message>
Update gh-pages to output generated at a3196b5
</commit_message>
<xml_diff>
--- a/上海-漫展信息.xlsx
+++ b/上海-漫展信息.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,7 +506,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1672</v>
+        <v>1673</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -644,7 +644,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -681,7 +681,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>淞虹路377号 长宁ArtPark大融城</t>
+          <t>剑川路1000号 龙湖上海闵行天街</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>369</v>
+        <v>390</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -707,7 +707,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202311/XmP03Vf31701070803044.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/tprwYGIB1705976768947.jpeg</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>527</v>
+        <v>543</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1158</v>
+        <v>1172</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -874,7 +874,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>908</v>
+        <v>931</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -920,7 +920,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2223</v>
+        <v>2224</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>631</v>
+        <v>648</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1020,7 +1020,7 @@
         </is>
       </c>
       <c r="H13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1058,7 +1058,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1104,7 +1104,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1150,7 +1150,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>637</v>
+        <v>672</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1196,7 +1196,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1242,7 +1242,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1288,7 +1288,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1291</v>
+        <v>1300</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1334,7 +1334,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1366,38 +1366,38 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>上海·魔都COS漫展-情人节专场AM01</t>
+          <t>上海·奇卡波利动漫嘉年华</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
+          <t>申滨路36号 虹桥丽宝广场</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2024.02.14 10:00-02.14 16:00</t>
+          <t>2024.02.14 10:00-02.14 17:00</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>84</v>
+        <v>32</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>48</t>
         </is>
       </c>
       <c r="H21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80691</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81260</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/aSdjV6Kw1704868345679.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/9OHovK2V1705978109130.jpeg</t>
         </is>
       </c>
     </row>
@@ -1407,30 +1407,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2024-02-16</t>
+          <t>2024-02-14</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>上海·第九届次元鹿角动漫游戏展</t>
+          <t>上海·魔都COS漫展-情人节专场AM01</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>盈浦街道淀山浦社区淀山湖大道851号青浦万达茂F3 万达汽车乐园(青浦万达茂店)</t>
+          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2024.02.16 11:00-02.17 18:00</t>
+          <t>2024.02.14 10:00-02.14 16:00</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>1205</v>
+        <v>90</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>49</t>
         </is>
       </c>
       <c r="H22" t="b">
@@ -1438,12 +1438,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80497</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80691</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/0duSXTQy1704423309244.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/aSdjV6Kw1704868345679.jpeg</t>
         </is>
       </c>
     </row>
@@ -1453,30 +1453,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2024-02-17</t>
+          <t>2024-02-16</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>上海·少女番only2.0</t>
+          <t>上海·第九届次元鹿角动漫游戏展</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>营口路699号(黄兴公园地铁站2号口旁) 花嫁丽舍</t>
+          <t>盈浦街道淀山浦社区淀山湖大道851号青浦万达茂F3 万达汽车乐园(青浦万达茂店)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2024.02.17 10:00-02.17 17:00</t>
+          <t>2024.02.16 11:00-02.17 18:00</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>189</v>
+        <v>1212</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>65</t>
         </is>
       </c>
       <c r="H23" t="b">
@@ -1484,12 +1484,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81148</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80497</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/j6eEZ18S1705657346664.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/0duSXTQy1704423309244.jpeg</t>
         </is>
       </c>
     </row>
@@ -1499,30 +1499,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2024-02-24</t>
+          <t>2024-02-17</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>上海·SISP动漫游戏嘉年华</t>
+          <t>上海·少女番only2.0</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>年家浜路518号 周浦万达广场</t>
+          <t>营口路699号(黄兴公园地铁站2号口旁) 花嫁丽舍</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2024.02.24 13:00-02.25 19:00</t>
+          <t>2024.02.17 10:00-02.17 17:00</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>111</v>
+        <v>231</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>80</t>
         </is>
       </c>
       <c r="H24" t="b">
@@ -1530,12 +1530,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80339</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81148</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202312/a8iuOufB1703832570508.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/j6eEZ18S1705657346664.jpeg</t>
         </is>
       </c>
     </row>
@@ -1550,38 +1550,38 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>上海·第三届燃梦BACG PRO游戏动漫展-原X铁X崩同好交流</t>
+          <t>上海·SISP动漫游戏嘉年华</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>盈浦街道淀山浦社区淀山湖大道851号青浦万达茂F3 万达汽车乐园(青浦万达茂店)</t>
+          <t>年家浜路518号 周浦万达广场</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2024.02.24 11:00-02.25 16:30</t>
+          <t>2024.02.24 13:00-02.25 19:00</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2471</v>
+        <v>116</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>48</t>
         </is>
       </c>
       <c r="H25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=77754</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80339</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202312/7eGZETK91701943985671.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202312/a8iuOufB1703832570508.jpeg</t>
         </is>
       </c>
     </row>
@@ -1596,38 +1596,38 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>上海·魔都元宵节漫展-COS为王</t>
+          <t>上海·第三届燃梦BACG PRO游戏动漫展-原X铁X崩同好交流</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
+          <t>盈浦街道淀山浦社区淀山湖大道851号青浦万达茂F3 万达汽车乐园(青浦万达茂店)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2024.02.24 10:00-02.25 16:00</t>
+          <t>2024.02.24 11:00-02.25 16:30</t>
         </is>
       </c>
       <c r="F26" t="n">
+        <v>2486</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="H26" t="b">
         <v>1</v>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>49</t>
-        </is>
-      </c>
-      <c r="H26" t="b">
-        <v>0</v>
-      </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81238</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=77754</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/KxQZPADR1705913896609.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202312/7eGZETK91701943985671.jpeg</t>
         </is>
       </c>
     </row>
@@ -1637,30 +1637,30 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2024-03-02</t>
+          <t>2024-02-24</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>上海·原神X星穹铁道ONLY</t>
+          <t>上海·魔都元宵节漫展-COS为王</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>逸仙路301号靠纪念路路口 上海宝丰联大酒店</t>
+          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2024.03.02 10:00-03.02 17:00</t>
+          <t>2024.02.24 10:00-02.25 16:00</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>246</v>
+        <v>4</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>49</t>
         </is>
       </c>
       <c r="H27" t="b">
@@ -1668,12 +1668,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80299</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81238</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202312/V0xu26Cl1703753850690.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/KxQZPADR1705913896609.jpeg</t>
         </is>
       </c>
     </row>
@@ -1683,26 +1683,26 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2024-03-03</t>
+          <t>2024-03-02</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>上海·怀旧番ONLY</t>
+          <t>上海·原神X星穹铁道ONLY</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>逸仙路270号  上海宝丰联大酒店</t>
+          <t>逸仙路301号靠纪念路路口 上海宝丰联大酒店</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2024.03.03 10:00-03.03 17:00</t>
+          <t>2024.03.02 10:00-03.02 17:00</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>124</v>
+        <v>252</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1714,12 +1714,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80575</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80299</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/y4uWdyPT1704700763902.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202312/V0xu26Cl1703753850690.jpeg</t>
         </is>
       </c>
     </row>
@@ -1729,30 +1729,30 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2024-03-09</t>
+          <t>2024-03-03</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>上海·S·CGE动漫游戏嘉年华</t>
+          <t>上海·怀旧番ONLY</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>军工路1076号 纪希片场(秀场)</t>
+          <t>逸仙路270号  上海宝丰联大酒店</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2024.03.09 10:00-03.10 17:00</t>
+          <t>2024.03.03 10:00-03.03 17:00</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>60</t>
         </is>
       </c>
       <c r="H29" t="b">
@@ -1760,12 +1760,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81173</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80575</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/TYA5FLkE1705891815532.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/y4uWdyPT1704700763902.jpeg</t>
         </is>
       </c>
     </row>
@@ -1780,38 +1780,38 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>上海·第五十三届燃梦星辰动漫嘉年华-随机宅舞</t>
+          <t>上海·S·CGE动漫游戏嘉年华</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>周家嘴路3608号 宝龙旭辉广场</t>
+          <t>军工路1076号 纪希片场(秀场)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2024.03.09 10:20-03.10 16:30</t>
+          <t>2024.03.09 10:00-03.10 17:00</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>70</t>
         </is>
       </c>
       <c r="H30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80571</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81173</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/SHH70VXN1704700240858.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/TYA5FLkE1705891815532.jpeg</t>
         </is>
       </c>
     </row>
@@ -1826,38 +1826,38 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>上海·青山刚昌ONLY【名侦探柯南&amp;魔术快斗】</t>
+          <t>上海·第五十三届燃梦星辰动漫嘉年华-随机宅舞</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>漕宝路1688号 诺宝中心酒店</t>
+          <t>周家嘴路3608号 宝龙旭辉广场</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2024.03.09 10:00-03.09 16:30</t>
+          <t>2024.03.09 10:20-03.10 16:30</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>865</v>
+        <v>43</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>58</t>
         </is>
       </c>
       <c r="H31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=76410</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80571</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202309/fVXMrcHy1693971682397.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/SHH70VXN1704700240858.jpeg</t>
         </is>
       </c>
     </row>
@@ -1867,30 +1867,30 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2024-03-16</t>
+          <t>2024-03-09</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>上海·坏孩纸物语の第33届动漫节之庄子篇</t>
+          <t>上海·青山刚昌ONLY【名侦探柯南&amp;魔术快斗】</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>中山北路3300号4楼L4001号 环球港上海世嘉都市乐园</t>
+          <t>漕宝路1688号 诺宝中心酒店</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2024.03.16 10:00-03.17 21:00</t>
+          <t>2024.03.09 10:00-03.09 16:30</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>16</v>
+        <v>875</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>73</t>
         </is>
       </c>
       <c r="H32" t="b">
@@ -1898,12 +1898,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81138</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=76410</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/jpr1lCt21705652306481.png</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202309/fVXMrcHy1693971682397.jpeg</t>
         </is>
       </c>
     </row>
@@ -1913,30 +1913,30 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2024-04-05</t>
+          <t>2024-03-16</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>上海·第四届次元鹿角动漫游戏展</t>
+          <t>上海·坏孩纸物语の第33届动漫节之庄子篇</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>顾村镇蕰川路6号 智慧湾科创园</t>
+          <t>中山北路3300号4楼L4001号 环球港上海世嘉都市乐园</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2024.04.05 10:00-04.06 17:00</t>
+          <t>2024.03.16 10:00-03.17 21:00</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="H33" t="b">
@@ -1944,12 +1944,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=78228</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81138</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202311/jgqIFxhx1699344723568.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/jpr1lCt21705652306481.png</t>
         </is>
       </c>
     </row>
@@ -1959,30 +1959,30 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2024-04-27</t>
+          <t>2024-04-05</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>上海·  第五十三届妖漫动漫游戏展</t>
+          <t>上海·第四届次元鹿角动漫游戏展</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>曹杨路1888号 复悦荟</t>
+          <t>顾村镇蕰川路6号 智慧湾科创园</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2024.04.27 10:00-04.27 17:00</t>
+          <t>2024.04.05 10:00-04.06 17:00</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>146</v>
+        <v>60</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>60</t>
         </is>
       </c>
       <c r="H34" t="b">
@@ -1990,12 +1990,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=78657</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=78228</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/tamNdgEN1705331335847.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202311/jgqIFxhx1699344723568.jpeg</t>
         </is>
       </c>
     </row>
@@ -2005,30 +2005,30 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2024-05-01</t>
+          <t>2024-04-27</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>上海·S·CGE动漫游戏嘉年华</t>
+          <t>上海·  第五十三届妖漫动漫游戏展</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>军工路1076号 纪希片场(秀场)</t>
+          <t>曹杨路1888号 复悦荟</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2024.05.01 10:00-05.02 17:00</t>
+          <t>2024.04.27 10:00-04.27 17:00</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2</v>
+        <v>148</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>80</t>
         </is>
       </c>
       <c r="H35" t="b">
@@ -2036,12 +2036,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81204</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=78657</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/nbFRULYe1705904589212.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/tamNdgEN1705331335847.jpeg</t>
         </is>
       </c>
     </row>
@@ -2056,25 +2056,25 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>上海·魔都野良神only</t>
+          <t>上海·S·CGE动漫游戏嘉年华</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>南京东路830号 第一百货</t>
+          <t>军工路1076号 纪希片场(秀场)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2024.05.01 10:00-05.01 17:00</t>
+          <t>2024.05.01 10:00-05.02 17:00</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>184</v>
+        <v>4</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>70</t>
         </is>
       </c>
       <c r="H36" t="b">
@@ -2082,12 +2082,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80321</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81204</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/KBlb0enU1704358750268.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/nbFRULYe1705904589212.jpeg</t>
         </is>
       </c>
     </row>
@@ -2097,41 +2097,87 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
+          <t>2024-05-01</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>上海·魔都野良神only</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>南京东路830号 第一百货</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2024.05.01 10:00-05.01 17:00</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>188</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="H37" t="b">
+        <v>0</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://show.bilibili.com/platform/detail.html?id=80321</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/KBlb0enU1704358750268.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
           <t>2024-05-05</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>上海·灌篮高手--青春永不散场</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>逸仙路1328弄 新业坊</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>2024.05.05 10:00-05.05 17:00</t>
         </is>
       </c>
-      <c r="F37" t="n">
-        <v>8</v>
-      </c>
-      <c r="G37" t="inlineStr">
+      <c r="F38" t="n">
+        <v>11</v>
+      </c>
+      <c r="G38" t="inlineStr">
         <is>
           <t>89</t>
         </is>
       </c>
-      <c r="H37" t="b">
-        <v>0</v>
-      </c>
-      <c r="I37" t="inlineStr">
+      <c r="H38" t="b">
+        <v>0</v>
+      </c>
+      <c r="I38" t="inlineStr">
         <is>
           <t>https://show.bilibili.com/platform/detail.html?id=80835</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="J38" t="inlineStr">
         <is>
           <t>//i1.hdslb.com/bfs/openplatform/202401/hdaVclFC1705301931054.jpeg</t>
         </is>
@@ -2148,7 +2194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2226,7 +2272,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -2345,30 +2391,30 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2024-01-23</t>
+          <t>2024-01-26</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>上海·七音阿卡莉 NANAOAKARI 2024 专场演出</t>
+          <t>上海·从Butter-Fly到夏目之爱してる —— “好想大声说爱你”动漫钢琴演奏会</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>嘉兴路街道瑞虹路188号瑞虹天地月亮湾3层 Modern Sky LAB摩登天空(瑞虹天地店)</t>
+          <t>丁香路425号 上海东方艺术中心</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2024.01.23 20:00-01.23 22:00</t>
+          <t>2024.01.26 19:30-01.26 21:30</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>91</v>
+        <v>163</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>已停售</t>
+          <t>80</t>
         </is>
       </c>
       <c r="H5" t="b">
@@ -2376,12 +2422,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79641</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=78418</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202312/CoNbgCpO1703644783043.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202311/GHpvkT5Y1699605760230.jpeg</t>
         </is>
       </c>
     </row>
@@ -2391,43 +2437,43 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2024-01-26</t>
+          <t>2024-01-27</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>上海·从Butter-Fly到夏目之爱してる —— “好想大声说爱你”动漫钢琴演奏会</t>
+          <t>上海·Azurock」Azurose ACG Cover Live</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>丁香路425号 上海东方艺术中心</t>
+          <t>愚园路1398号 育音堂音乐公园</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2024.01.26 19:30-01.26 21:30</t>
+          <t>2024.01.27 19:00-01.27 21:30</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>161</v>
+        <v>60</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>88</t>
         </is>
       </c>
       <c r="H6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=78418</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80277</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202311/GHpvkT5Y1699605760230.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202312/5d6O1Rf11703742965244.png</t>
         </is>
       </c>
     </row>
@@ -2442,38 +2488,38 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>上海·Azurock」Azurose ACG Cover Live</t>
+          <t>上海·日本原版《数码宝贝舞台剧：游乐园之谜》</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>愚园路1398号 育音堂音乐公园</t>
+          <t>茂名南路57号近长乐路 上海兰心大戏院</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2024.01.27 19:00-01.27 21:30</t>
+          <t>2024.01.27 15:30-01.27 20:55</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>120</t>
         </is>
       </c>
       <c r="H7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80277</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=79783</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202312/5d6O1Rf11703742965244.png</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202312/S6nZ327b1702534484951.jpeg</t>
         </is>
       </c>
     </row>
@@ -2488,25 +2534,25 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>上海·日本原版《数码宝贝舞台剧：游乐园之谜》</t>
+          <t>上海•Risa Yuzuki 1st ONEMAN LIVE 「Future Interlink」 追加公演</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>茂名南路57号近长乐路 上海兰心大戏院</t>
+          <t>愚园路1250号 新歌空间</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2024.01.27 15:30-01.27 20:55</t>
+          <t>2024.01.27 18:30-01.27 21:00</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>30</v>
+        <v>298</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>278</t>
         </is>
       </c>
       <c r="H8" t="b">
@@ -2514,12 +2560,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79783</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=77773</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202312/S6nZ327b1702534484951.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202310/XKKYWAk51698315607196.png</t>
         </is>
       </c>
     </row>
@@ -2529,30 +2575,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2024-01-27</t>
+          <t>2024-02-02</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>上海•Risa Yuzuki 1st ONEMAN LIVE 「Future Interlink」 追加公演</t>
+          <t>上海·次元LAB 二次元电音节</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>愚园路1250号 新歌空间</t>
+          <t>中兴路1683号金融街购物中心L3-27 蜚声上海Livehouse</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2024.01.27 18:30-01.27 21:00</t>
+          <t>2024.02.02 12:30-02.02 21:00</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>298</v>
+        <v>631</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>380</t>
         </is>
       </c>
       <c r="H9" t="b">
@@ -2560,12 +2606,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=77773</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80128</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202310/XKKYWAk51698315607196.png</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202312/DEW1XYty1703226993965.jpeg</t>
         </is>
       </c>
     </row>
@@ -2575,43 +2621,43 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2024-02-02</t>
+          <t>2024-02-04</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>上海·次元LAB 二次元电音节</t>
+          <t>上海·触手猴钢琴巡演·marasy piano live tour『生音』上海站·Powered by 东方弹幕神乐失落幻想</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>中兴路1683号金融街购物中心L3-27 蜚声上海Livehouse</t>
+          <t>丁香路425号(上海科技馆地铁站1号口步行460米) 上海东方艺术中心音乐厅</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2024.02.02 12:30-02.02 21:00</t>
+          <t>2024.02.04 19:30-02.04 21:00</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>620</v>
+        <v>339</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>380</t>
+          <t>280</t>
         </is>
       </c>
       <c r="H10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80128</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80734</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202312/DEW1XYty1703226993965.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/IcjPp0TE1704951328918.jpeg</t>
         </is>
       </c>
     </row>
@@ -2621,30 +2667,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2024-02-04</t>
+          <t>2024-02-14</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>上海·触手猴钢琴巡演·marasy piano live tour『生音』上海站·Powered by 东方弹幕神乐失落幻想</t>
+          <t>上海·【情人节特辑】《那年我们》记忆重启韩剧经典OST音乐会《请回答1988》《来自星星的你》</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>丁香路425号(上海科技馆地铁站1号口步行460米) 上海东方艺术中心音乐厅</t>
+          <t>牛庄路704号 中国大戏院</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2024.02.04 19:30-02.04 21:00</t>
+          <t>2024.02.14 19:30-02.14 21:00</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>329</v>
+        <v>2</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>已停售</t>
         </is>
       </c>
       <c r="H11" t="b">
@@ -2652,12 +2698,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80734</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80615</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/IcjPp0TE1704951328918.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/5DDVhKcO1704767761361.png</t>
         </is>
       </c>
     </row>
@@ -2667,30 +2713,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2024-02-14</t>
+          <t>2024-02-24</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>上海·【情人节特辑】《那年我们》记忆重启韩剧经典OST音乐会《请回答1988》《来自星星的你》</t>
+          <t>上海·《哈利的魔法世界》动漫视听音乐会</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>牛庄路704号 中国大戏院</t>
+          <t>都市路4889号（莘庄地铁站南广场） 上海保利城市剧院</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2024.02.14 19:30-02.14 21:00</t>
+          <t>2024.02.24 14:30-02.24 16:00</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>已停售</t>
+          <t>158</t>
         </is>
       </c>
       <c r="H12" t="b">
@@ -2698,12 +2744,12 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80615</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80639</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/5DDVhKcO1704767761361.png</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/dp013A4p1704783993628.png</t>
         </is>
       </c>
     </row>
@@ -2713,30 +2759,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2024-02-24</t>
+          <t>2024-02-25</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>上海·《哈利的魔法世界》动漫视听音乐会</t>
+          <t>上海·青山吉能见面会</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>都市路4889号（莘庄地铁站南广场） 上海保利城市剧院</t>
+          <t>虹许路731号4号楼 THE BOXX•城市乐园</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2024.02.24 14:30-02.24 16:00</t>
+          <t>2024.02.25 14:30-02.25 19:30</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>5</v>
+        <v>200</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>380</t>
         </is>
       </c>
       <c r="H13" t="b">
@@ -2744,12 +2790,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80639</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80142</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/dp013A4p1704783993628.png</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202312/1npuHFBM1703231674558.jpeg</t>
         </is>
       </c>
     </row>
@@ -2759,43 +2805,43 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2024-02-25</t>
+          <t>2024-03-02</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>上海·青山吉能见面会</t>
+          <t>上海·2024藤田玲上海粉丝见面会</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>虹许路731号4号楼 THE BOXX•城市乐园</t>
+          <t>宜昌路179号 万代南梦宫上海文化中心</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2024.02.25 14:30-02.25 19:30</t>
+          <t>2024.03.02 12:30-03.02 19:40</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>199</v>
+        <v>9</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>380</t>
+          <t>580</t>
         </is>
       </c>
       <c r="H14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80142</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80993</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202312/1npuHFBM1703231674558.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/Vm6ntgVd1705548188785.png</t>
         </is>
       </c>
     </row>
@@ -2810,7 +2856,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>上海·2024藤田玲上海粉丝见面会</t>
+          <t>上海·小山百代2024上海粉丝见面会</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2820,15 +2866,15 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2024.03.02 12:30-03.02 19:40</t>
+          <t>2024.03.02 13:00-03.02 20:00</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>5</v>
+        <v>235</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>580</t>
+          <t>380</t>
         </is>
       </c>
       <c r="H15" t="b">
@@ -2836,12 +2882,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80993</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80924</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/Vm6ntgVd1705548188785.png</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/FpA9OkKy1705467080070.jpeg</t>
         </is>
       </c>
     </row>
@@ -2870,7 +2916,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -2897,43 +2943,43 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2024-03-02</t>
+          <t>2024-03-09</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>上海·小山百代2024上海粉丝见面会</t>
+          <t>上海·《挪威的森林》—摇滚情歌之夜演唱会</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>宜昌路179号 万代南梦宫上海文化中心</t>
+          <t>南京西路1376号 上海商城剧院</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2024.03.02 13:00-03.02 20:00</t>
+          <t>2024.03.09 19:30-03.09 21:00</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>226</v>
+        <v>0</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>380</t>
+          <t>72</t>
         </is>
       </c>
       <c r="H17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80924</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81241</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/FpA9OkKy1705467080070.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/1FJ0Fj5m1705915336335.jpeg</t>
         </is>
       </c>
     </row>
@@ -2948,7 +2994,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>上海·《挪威的森林》—摇滚情歌之夜演唱会</t>
+          <t>上海·爱乐之城音乐会</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2958,7 +3004,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2024.03.09 19:30-03.09 21:00</t>
+          <t>2024.03.09 14:00-03.09 15:30</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -2966,7 +3012,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>60</t>
         </is>
       </c>
       <c r="H18" t="b">
@@ -2974,12 +3020,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81241</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81289</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/1FJ0Fj5m1705915336335.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/ZZXtDrwZ1705996679699.jpeg</t>
         </is>
       </c>
     </row>
@@ -3008,7 +3054,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -3100,7 +3146,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>380</v>
+        <v>471</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -3173,30 +3219,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2024-03-21</t>
+          <t>2024-03-17</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>上海·春卷饭 十周年  2024  专场演出</t>
+          <t>上海·遇见新海诚--帝玖「这次一定」室内乐ACG音乐会</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>嘉兴路街道瑞虹路188号瑞虹天地月亮湾3层 Modern Sky LAB摩登天空(瑞虹天地店)</t>
+          <t>延安东路523号 凯迪拉克·上海音乐厅</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2024.03.21 20:00-03.21 22:00</t>
+          <t>2024.03.17 14:00-03.17 16:00</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>271</v>
+        <v>5</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>480</t>
+          <t>80</t>
         </is>
       </c>
       <c r="H23" t="b">
@@ -3204,12 +3250,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81190</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81258</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/ho9rIMg21705894649801.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/eysvN81k1705977896972.jpeg</t>
         </is>
       </c>
     </row>
@@ -3219,30 +3265,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2024-03-30</t>
+          <t>2024-03-21</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>上海· TRUE（唐沢美帆）上海动漫交响音乐会</t>
+          <t>上海·春卷饭 十周年  2024  专场演出</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>丁香路425号 上海东方艺术中心</t>
+          <t>嘉兴路街道瑞虹路188号瑞虹天地月亮湾3层 Modern Sky LAB摩登天空(瑞虹天地店)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2024.03.30 19:30-03.30 21:00</t>
+          <t>2024.03.21 20:00-03.21 22:00</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>140</v>
+        <v>349</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>280</t>
+          <t>480</t>
         </is>
       </c>
       <c r="H24" t="b">
@@ -3250,12 +3296,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80906</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81190</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/FaJbLvS51705401178235.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/ho9rIMg21705894649801.jpeg</t>
         </is>
       </c>
     </row>
@@ -3265,43 +3311,43 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2024-04-06</t>
+          <t>2024-03-30</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>上海·从Butter-Fly到夏目之爱してる —— “好想大声说爱你”动漫钢琴演奏会</t>
+          <t>上海· TRUE（唐沢美帆）上海动漫交响音乐会</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>复兴中路1380号 捷豹上海交响音乐厅</t>
+          <t>丁香路425号 上海东方艺术中心</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2024.04.06 19:30-04.06 21:30</t>
+          <t>2024.03.30 19:30-03.30 21:00</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>280</t>
         </is>
       </c>
       <c r="H25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80050</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80906</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202312/0iJP3TY61703056498448.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/FaJbLvS51705401178235.jpeg</t>
         </is>
       </c>
     </row>
@@ -3311,26 +3357,26 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2024-04-13</t>
+          <t>2024-04-06</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>上海·《四月是你的谎言》——“公生”与“薰”的钢琴小提琴唯美经典音乐集</t>
+          <t>上海·从Butter-Fly到夏目之爱してる —— “好想大声说爱你”动漫钢琴演奏会</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>丁香路425号 上海东方艺术中心</t>
+          <t>复兴中路1380号 捷豹上海交响音乐厅</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2024.04.13 19:30-04.13 21:30</t>
+          <t>2024.04.06 19:30-04.06 21:30</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>171</v>
+        <v>10</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -3342,12 +3388,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=78667</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80050</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202311/bTP7w6GD1700130122940.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202312/0iJP3TY61703056498448.jpeg</t>
         </is>
       </c>
     </row>
@@ -3357,26 +3403,26 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2024-04-20</t>
+          <t>2024-04-13</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>上海·Laurent Coulondre“心动巴黎”2024中国巡回音乐会</t>
+          <t>上海·《四月是你的谎言》——“公生”与“薰”的钢琴小提琴唯美经典音乐集</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>汾阳路20号上海音乐学院内 上海贺绿汀音乐厅</t>
+          <t>丁香路425号 上海东方艺术中心</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2024.04.20 19:30-04.20 21:30</t>
+          <t>2024.04.13 19:30-04.13 21:30</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>3</v>
+        <v>172</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -3384,16 +3430,16 @@
         </is>
       </c>
       <c r="H27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81135</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=78667</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/wXDdS5ap1705651730828.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202311/bTP7w6GD1700130122940.jpeg</t>
         </is>
       </c>
     </row>
@@ -3403,41 +3449,87 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>2024-04-20</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>上海·Laurent Coulondre“心动巴黎”2024中国巡回音乐会</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>汾阳路20号上海音乐学院内 上海贺绿汀音乐厅</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2024.04.20 19:30-04.20 21:30</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>3</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="H28" t="b">
+        <v>0</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://show.bilibili.com/platform/detail.html?id=81135</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/wXDdS5ap1705651730828.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>2024-04-26</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>上海· 夏川里美 2024 巡回演唱会 出道 25 周年纪念专场</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>东大名路889号 友邦大剧院</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>2024.04.26 19:30-04.26 21:30</t>
         </is>
       </c>
-      <c r="F28" t="n">
-        <v>10</v>
-      </c>
-      <c r="G28" t="inlineStr">
+      <c r="F29" t="n">
+        <v>11</v>
+      </c>
+      <c r="G29" t="inlineStr">
         <is>
           <t>280</t>
         </is>
       </c>
-      <c r="H28" t="b">
-        <v>0</v>
-      </c>
-      <c r="I28" t="inlineStr">
+      <c r="H29" t="b">
+        <v>0</v>
+      </c>
+      <c r="I29" t="inlineStr">
         <is>
           <t>https://show.bilibili.com/platform/detail.html?id=81139</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>//i2.hdslb.com/bfs/openplatform/202401/0Fj4cYOH1705652393930.jpeg</t>
         </is>
@@ -3624,7 +3716,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -3670,7 +3762,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1984</v>
+        <v>1995</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -3716,7 +3808,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2082</v>
+        <v>2101</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -3762,7 +3854,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>820</v>
+        <v>824</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -3804,11 +3896,11 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2024.01.06 00:00-01.31 23:59</t>
+          <t>2024.01.06 00:00-02.29 23:59</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>703</v>
+        <v>726</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -3899,30 +3991,30 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2023-01-12</t>
+          <t>2023-10-16</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>上海·日漫咖啡体验</t>
+          <t>上海·古影文化《1941·新和医院》大型沉浸式互动剧场</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>虹桥路1438号高岛屋百货6楼 OASIS书吧</t>
+          <t>金玉路2号 古影沉浸式互动游戏剧场</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2023.01.12 10:00-2024.02.29 22:00</t>
+          <t>2023.10.16 10:00-2024.10.15 21:00</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1726</v>
+        <v>69</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>996</t>
         </is>
       </c>
       <c r="H2" t="b">
@@ -3930,12 +4022,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=70666</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=77530</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202106/okF9H2Uj1623911727887.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202310/JqP3lHJt1698030195136.jpeg</t>
         </is>
       </c>
     </row>
@@ -3945,30 +4037,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2023-10-16</t>
+          <t>2023-10-25</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>上海·古影文化《1941·新和医院》大型沉浸式互动剧场</t>
+          <t>上海·方块大战（豫园店）</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>金玉路2号 古影沉浸式互动游戏剧场</t>
+          <t>丽水路88号2楼213 城隍庙第一购物中心</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2023.10.16 10:00-2024.10.15 21:00</t>
+          <t>2023.10.25 10:00-2024.10.20 21:00</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>69</v>
+        <v>38</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>996</t>
+          <t>49</t>
         </is>
       </c>
       <c r="H3" t="b">
@@ -3976,12 +4068,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=77530</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=79057</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202310/JqP3lHJt1698030195136.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202312/ASamaqBx1701419480253.jpeg</t>
         </is>
       </c>
     </row>
@@ -3991,30 +4083,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2023-10-25</t>
+          <t>2023-11-02</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>上海·方块大战（豫园店）</t>
+          <t>上海·Hello Kitty Cosmos 50周年光影特展</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>丽水路88号2楼213 城隍庙第一购物中心</t>
+          <t>漕宝路3055号 宝龙美术馆</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2023.10.25 10:00-2024.10.20 21:00</t>
+          <t>2023.11.02 10:00-2024.01.28 18:00</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>36</v>
+        <v>121</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>139</t>
         </is>
       </c>
       <c r="H4" t="b">
@@ -4022,12 +4114,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79057</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=77862</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202312/ASamaqBx1701419480253.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202310/QnmD4yOd1698652192047.jpeg</t>
         </is>
       </c>
     </row>
@@ -4037,30 +4129,30 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2023-11-02</t>
+          <t>2023-12-01</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>上海·Hello Kitty Cosmos 50周年光影特展</t>
+          <t>上海·2023《蔚蓝档案》x  萌果酱谷子咖啡</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>漕宝路3055号 宝龙美术馆</t>
+          <t>南京东路340号百联ZX 萌果酱谷子咖啡（百联）</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2023.11.02 10:00-2024.01.28 18:00</t>
+          <t>2023.12.01 00:00-2024.01.31 23:59</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>120</v>
+        <v>1995</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>30</t>
         </is>
       </c>
       <c r="H5" t="b">
@@ -4068,12 +4160,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=77862</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=79005</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202310/QnmD4yOd1698652192047.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202311/02P8eD3Z1700821985538.jpeg</t>
         </is>
       </c>
     </row>
@@ -4083,26 +4175,26 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2023-12-01</t>
+          <t>2023-12-06</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>上海·2023《蔚蓝档案》x  萌果酱谷子咖啡</t>
+          <t>上海·「咒术回战  × animate cafe」</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>南京东路340号百联ZX 萌果酱谷子咖啡（百联）</t>
+          <t>西藏北路198号大悦城北座8楼N809-1 animate cafe上海店</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2023.12.01 00:00-2024.01.31 23:59</t>
+          <t>2023.12.06 00:00-2024.02.27 23:59</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1984</v>
+        <v>2101</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -4114,12 +4206,12 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79005</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=79292</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202311/02P8eD3Z1700821985538.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/LyD46Kty1705488020552.jpeg</t>
         </is>
       </c>
     </row>
@@ -4129,30 +4221,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2023-12-06</t>
+          <t>2023-12-22</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>上海·「咒术回战  × animate cafe」</t>
+          <t>上海·新海诚导演作品《铃芽之旅》展 丨 购票抽新海诚见面会门票丨 超限定复刻原画发售</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>西藏北路198号大悦城北座8楼N809-1 animate cafe上海店</t>
+          <t>湖滨路168号 上海无限极荟购物中心</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2023.12.06 00:00-2024.02.27 23:59</t>
+          <t>2023.12.22 10:00-2024.02.16 22:00</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2082</v>
+        <v>1673</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>55</t>
         </is>
       </c>
       <c r="H7" t="b">
@@ -4160,12 +4252,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79292</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=79166</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/LyD46Kty1705488020552.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202311/MjTiIYlk1701242361853.jpeg</t>
         </is>
       </c>
     </row>
@@ -4175,30 +4267,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2023-12-22</t>
+          <t>2023-12-25</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>上海·新海诚导演作品《铃芽之旅》展 丨 购票抽新海诚见面会门票丨 超限定复刻原画发售</t>
+          <t>上海·爱乐汇“浪漫经典·一生必听”永恒精选2023烛光音乐会</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>湖滨路168号 上海无限极荟购物中心</t>
+          <t>南京西路1376号 上海商城剧院</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2023.12.22 10:00-2024.02.16 22:00</t>
+          <t>2023.12.25 19:30-2024.02.27 21:00</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>1672</v>
+        <v>24</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>90</t>
         </is>
       </c>
       <c r="H8" t="b">
@@ -4206,12 +4298,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79166</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80057</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202311/MjTiIYlk1701242361853.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202312/AeWGG9Rk1703131189224.jpeg</t>
         </is>
       </c>
     </row>
@@ -4221,12 +4313,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2023-12-25</t>
+          <t>2023-12-27</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>上海·爱乐汇“浪漫经典·一生必听”永恒精选2023烛光音乐会</t>
+          <t>上海·爱乐汇《天空之城》久石让&amp;宫崎骏动漫经典音乐作品演奏会</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -4236,11 +4328,11 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2023.12.25 19:30-2024.02.27 21:00</t>
+          <t>2023.12.27 19:30-2024.02.03 12:00</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -4252,12 +4344,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80057</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80103</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202312/AeWGG9Rk1703131189224.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202312/2h2tIq7l1703144874867.png</t>
         </is>
       </c>
     </row>
@@ -4267,30 +4359,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2023-12-27</t>
+          <t>2023-12-31</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>上海·爱乐汇《天空之城》久石让&amp;宫崎骏动漫经典音乐作品演奏会</t>
+          <t>上海·次元波板糖×时光代理人「锦瑟华年主题快闪店」</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>南京西路1376号 上海商城剧院</t>
+          <t>西藏北路166静安大悦城北座6楼611号 次元波板糖</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2023.12.27 19:30-2024.02.03 12:00</t>
+          <t>2023.12.31 00:00-2024.01.29 23:59</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>42</v>
+        <v>824</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>30</t>
         </is>
       </c>
       <c r="H10" t="b">
@@ -4298,12 +4390,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80103</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=79972</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202312/2h2tIq7l1703144874867.png</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202312/z7bFCMqM1702972063289.png</t>
         </is>
       </c>
     </row>
@@ -4313,30 +4405,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2023-12-31</t>
+          <t>2024-01-06</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>上海·次元波板糖×时光代理人「锦瑟华年主题快闪店」</t>
+          <t>上海·罗小黑 x HAPPY ZOO主题Cafe</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>西藏北路166静安大悦城北座6楼611号 次元波板糖</t>
+          <t>南京东路340号 百联zx创趣场</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2023.12.31 00:00-2024.01.29 23:59</t>
+          <t>2024.01.06 00:00-02.29 23:59</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>820</v>
+        <v>726</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H11" t="b">
@@ -4344,12 +4436,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79972</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80171</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202312/z7bFCMqM1702972063289.png</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202312/chPePM8d1703485388734.png</t>
         </is>
       </c>
     </row>
@@ -4359,43 +4451,43 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2024-01-06</t>
+          <t>2024-01-26</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>上海·罗小黑 x HAPPY ZOO主题Cafe</t>
+          <t>上海·从Butter-Fly到夏目之爱してる —— “好想大声说爱你”动漫钢琴演奏会</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>南京东路340号 百联zx创趣场</t>
+          <t>丁香路425号 上海东方艺术中心</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2024.01.06 00:00-01.31 23:59</t>
+          <t>2024.01.26 19:30-01.26 21:30</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>703</v>
+        <v>163</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>80</t>
         </is>
       </c>
       <c r="H12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80171</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=78418</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202312/chPePM8d1703485388734.png</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202311/GHpvkT5Y1699605760230.jpeg</t>
         </is>
       </c>
     </row>
@@ -4405,43 +4497,43 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2024-01-26</t>
+          <t>2024-01-27</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>上海·从Butter-Fly到夏目之爱してる —— “好想大声说爱你”动漫钢琴演奏会</t>
+          <t>上海·25时主题同人茶会</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>丁香路425号 上海东方艺术中心</t>
+          <t>沪太路3100号 尚大国际</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2024.01.26 19:30-01.26 21:30</t>
+          <t>2024.01.27 12:00-01.27 18:00</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>161</v>
+        <v>131</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>68</t>
         </is>
       </c>
       <c r="H13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=78418</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80548</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202311/GHpvkT5Y1699605760230.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/dQ4DrxCk1704683144116.png</t>
         </is>
       </c>
     </row>
@@ -4456,25 +4548,25 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>上海·25时主题同人茶会</t>
+          <t>上海·Azurock」Azurose ACG Cover Live</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>沪太路3100号 尚大国际</t>
+          <t>愚园路1398号 育音堂音乐公园</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2024.01.27 12:00-01.27 18:00</t>
+          <t>2024.01.27 19:00-01.27 21:30</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>126</v>
+        <v>60</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>88</t>
         </is>
       </c>
       <c r="H14" t="b">
@@ -4482,12 +4574,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80548</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80277</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/dQ4DrxCk1704683144116.png</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202312/5d6O1Rf11703742965244.png</t>
         </is>
       </c>
     </row>
@@ -4502,25 +4594,25 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>上海·Azurock」Azurose ACG Cover Live</t>
+          <t>上海·SISPmini动漫游戏嘉年华</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>愚园路1398号 育音堂音乐公园</t>
+          <t>剑川路1000号 龙湖上海闵行天街</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2024.01.27 19:00-01.27 21:30</t>
+          <t>2024.01.27 13:00-01.28 19:00</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>59</v>
+        <v>390</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>48</t>
         </is>
       </c>
       <c r="H15" t="b">
@@ -4528,12 +4620,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80277</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=79046</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202312/5d6O1Rf11703742965244.png</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/tprwYGIB1705976768947.jpeg</t>
         </is>
       </c>
     </row>
@@ -4548,25 +4640,25 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>上海·SISPmini动漫游戏嘉年华</t>
+          <t>上海·同好召集令火影only</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>淞虹路377号 长宁ArtPark大融城</t>
+          <t>市真南路1199弄1号 智创TOP综合体产城</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2024.01.27 13:00-01.28 19:00</t>
+          <t>2024.01.27 10:00-01.28 18:00</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>369</v>
+        <v>543</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>78</t>
         </is>
       </c>
       <c r="H16" t="b">
@@ -4574,12 +4666,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79046</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80284</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202311/XmP03Vf31701070803044.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/9xGb6MXN1704183627126.jpeg</t>
         </is>
       </c>
     </row>
@@ -4594,25 +4686,25 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>上海·同好召集令火影only</t>
+          <t>上海·咒术only-幽暗之森1.0</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>市真南路1199弄1号 智创TOP综合体产城</t>
+          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2024.01.27 10:00-01.28 18:00</t>
+          <t>2024.01.27 10:00-01.27 16:00</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>527</v>
+        <v>251</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>59</t>
         </is>
       </c>
       <c r="H17" t="b">
@@ -4620,12 +4712,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80284</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80045</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/9xGb6MXN1704183627126.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202312/hUfcrw3y1703055422885.jpeg</t>
         </is>
       </c>
     </row>
@@ -4640,38 +4732,38 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>上海·咒术only-幽暗之森1.0</t>
+          <t>上海·日本原版《数码宝贝舞台剧：游乐园之谜》</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
+          <t>茂名南路57号近长乐路 上海兰心大戏院</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2024.01.27 10:00-01.27 16:00</t>
+          <t>2024.01.27 15:30-01.27 20:55</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>248</v>
+        <v>31</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>120</t>
         </is>
       </c>
       <c r="H18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80045</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=79783</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202312/hUfcrw3y1703055422885.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202312/S6nZ327b1702534484951.jpeg</t>
         </is>
       </c>
     </row>
@@ -4686,38 +4778,38 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>上海·日本原版《数码宝贝舞台剧：游乐园之谜》</t>
+          <t>上海·第八届次元鹿角动漫游戏展</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>茂名南路57号近长乐路 上海兰心大戏院</t>
+          <t>吴中路1588号上海爱琴海购物中心F4 竞梦元宇宙</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2024.01.27 15:30-01.27 20:55</t>
+          <t>2024.01.27 10:00-01.28 21:00</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>30</v>
+        <v>1172</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>68</t>
         </is>
       </c>
       <c r="H19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79783</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80979</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202312/S6nZ327b1702534484951.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/xPOF923U1705545223366.jpeg</t>
         </is>
       </c>
     </row>
@@ -4732,25 +4824,25 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>上海·第八届次元鹿角动漫游戏展</t>
+          <t>上海·魔都寒假漫展-CF01</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>吴中路1588号上海爱琴海购物中心F4 竞梦元宇宙</t>
+          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2024.01.27 10:00-01.28 21:00</t>
+          <t>2024.01.27 10:00-01.28 16:00</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1158</v>
+        <v>931</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>49</t>
         </is>
       </c>
       <c r="H20" t="b">
@@ -4758,12 +4850,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80979</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80204</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/xPOF923U1705545223366.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202312/eK96fdcg1703573110264.jpeg</t>
         </is>
       </c>
     </row>
@@ -4778,38 +4870,38 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>上海·魔都寒假漫展-CF01</t>
+          <t>上海•Risa Yuzuki 1st ONEMAN LIVE 「Future Interlink」 追加公演</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
+          <t>愚园路1250号 新歌空间</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2024.01.27 10:00-01.28 16:00</t>
+          <t>2024.01.27 18:30-01.27 21:00</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>909</v>
+        <v>298</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>278</t>
         </is>
       </c>
       <c r="H21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80204</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=77773</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202312/eK96fdcg1703573110264.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202310/XKKYWAk51698315607196.png</t>
         </is>
       </c>
     </row>
@@ -4819,43 +4911,43 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2024-01-27</t>
+          <t>2024-01-28</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>上海•Risa Yuzuki 1st ONEMAN LIVE 「Future Interlink」 追加公演</t>
+          <t>上海 ·WOW潮元原神x星铁主题二次元狂欢派对</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>愚园路1250号 新歌空间</t>
+          <t>政通路189号五角场万达广场C栋 元气森林livehouse</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2024.01.27 18:30-01.27 21:00</t>
+          <t>2024.01.28 14:00-01.28 19:00</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>298</v>
+        <v>428</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>278</t>
+          <t>129</t>
         </is>
       </c>
       <c r="H22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=77773</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80167</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202310/XKKYWAk51698315607196.png</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/QTp32HEM1705028548091.jpeg</t>
         </is>
       </c>
     </row>
@@ -4865,30 +4957,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2024-01-28</t>
+          <t>2024-01-31</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>上海 ·WOW潮元原神x星铁主题二次元狂欢派对</t>
+          <t>上海·寻迹冬日LOVELIVE同好会</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>政通路189号五角场万达广场C栋 元气森林livehouse</t>
+          <t>愚园路1250号 新歌空间</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2024.01.28 14:00-01.28 19:00</t>
+          <t>2024.01.31 11:30-01.31 17:00</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>420</v>
+        <v>186</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>129</t>
+          <t>83</t>
         </is>
       </c>
       <c r="H23" t="b">
@@ -4896,12 +4988,12 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80167</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=79332</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/QTp32HEM1705028548091.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202312/Ewreg1JT1701677993728.jpeg</t>
         </is>
       </c>
     </row>
@@ -4911,43 +5003,43 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2024-01-31</t>
+          <t>2024-02-02</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>上海·寻迹冬日LOVELIVE同好会</t>
+          <t>上海·次元LAB 二次元电音节</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>愚园路1250号 新歌空间</t>
+          <t>中兴路1683号金融街购物中心L3-27 蜚声上海Livehouse</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2024.01.31 11:30-01.31 17:00</t>
+          <t>2024.02.02 12:30-02.02 21:00</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>183</v>
+        <v>631</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>380</t>
         </is>
       </c>
       <c r="H24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79332</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80128</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202312/Ewreg1JT1701677993728.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202312/DEW1XYty1703226993965.jpeg</t>
         </is>
       </c>
     </row>
@@ -4957,43 +5049,43 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2024-02-02</t>
+          <t>2024-02-03</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>上海·次元LAB 二次元电音节</t>
+          <t>上海·Coser迎春动漫展</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>中兴路1683号金融街购物中心L3-27 蜚声上海Livehouse</t>
+          <t>海潮路133号B1 JUMP工坊</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2024.02.02 12:30-02.02 21:00</t>
+          <t>2024.02.03 10:00-02.04 17:00</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>620</v>
+        <v>672</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>380</t>
+          <t>60</t>
         </is>
       </c>
       <c r="H25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80128</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80646</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202312/DEW1XYty1703226993965.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/4WVkFc4d1704787729064.jpeg</t>
         </is>
       </c>
     </row>
@@ -5008,25 +5100,25 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>上海·Coser迎春动漫展</t>
+          <t>上海·偶像梦幻祭红白歌合战Only</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>海潮路133号B1 JUMP工坊</t>
+          <t>虹许路731号4号楼 THE BOXX•城市乐园</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2024.02.03 10:00-02.04 17:00</t>
+          <t>2024.02.03 13:30-02.03 22:00</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>637</v>
+        <v>30</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>88</t>
         </is>
       </c>
       <c r="H26" t="b">
@@ -5034,12 +5126,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80646</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81199</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/4WVkFc4d1704787729064.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/C7E7svbZ1705903245860.jpeg</t>
         </is>
       </c>
     </row>
@@ -5049,30 +5141,30 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2024-02-03</t>
+          <t>2024-02-04</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>上海·偶像梦幻祭红白歌合战Only</t>
+          <t>上海·触手猴钢琴巡演·marasy piano live tour『生音』上海站·Powered by 东方弹幕神乐失落幻想</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>虹许路731号4号楼 THE BOXX•城市乐园</t>
+          <t>丁香路425号(上海科技馆地铁站1号口步行460米) 上海东方艺术中心音乐厅</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2024.02.03 13:30-02.03 22:00</t>
+          <t>2024.02.04 19:30-02.04 21:00</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>13</v>
+        <v>339</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>280</t>
         </is>
       </c>
       <c r="H27" t="b">
@@ -5080,12 +5172,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81199</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80734</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/C7E7svbZ1705903245860.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/IcjPp0TE1704951328918.jpeg</t>
         </is>
       </c>
     </row>
@@ -5114,7 +5206,7 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -5141,30 +5233,30 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2024-02-14</t>
+          <t>2024-02-16</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>上海·魔都COS漫展-情人节专场AM01</t>
+          <t>上海·第九届次元鹿角动漫游戏展</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
+          <t>盈浦街道淀山浦社区淀山湖大道851号青浦万达茂F3 万达汽车乐园(青浦万达茂店)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2024.02.14 10:00-02.14 16:00</t>
+          <t>2024.02.16 11:00-02.17 18:00</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>84</v>
+        <v>1212</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>65</t>
         </is>
       </c>
       <c r="H29" t="b">
@@ -5172,12 +5264,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80691</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80497</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/aSdjV6Kw1704868345679.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/0duSXTQy1704423309244.jpeg</t>
         </is>
       </c>
     </row>
@@ -5187,30 +5279,30 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2024-02-16</t>
+          <t>2024-02-17</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>上海·第九届次元鹿角动漫游戏展</t>
+          <t>上海·少女番only2.0</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>盈浦街道淀山浦社区淀山湖大道851号青浦万达茂F3 万达汽车乐园(青浦万达茂店)</t>
+          <t>营口路699号(黄兴公园地铁站2号口旁) 花嫁丽舍</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2024.02.16 11:00-02.17 18:00</t>
+          <t>2024.02.17 10:00-02.17 17:00</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>1205</v>
+        <v>231</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>80</t>
         </is>
       </c>
       <c r="H30" t="b">
@@ -5218,12 +5310,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80497</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81148</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/0duSXTQy1704423309244.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/j6eEZ18S1705657346664.jpeg</t>
         </is>
       </c>
     </row>
@@ -5233,30 +5325,30 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2024-02-17</t>
+          <t>2024-02-24</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>上海·少女番only2.0</t>
+          <t>上海·SISP动漫游戏嘉年华</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>营口路699号(黄兴公园地铁站2号口旁) 花嫁丽舍</t>
+          <t>年家浜路518号 周浦万达广场</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2024.02.17 10:00-02.17 17:00</t>
+          <t>2024.02.24 13:00-02.25 19:00</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>189</v>
+        <v>116</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>48</t>
         </is>
       </c>
       <c r="H31" t="b">
@@ -5264,12 +5356,12 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81148</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80339</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/j6eEZ18S1705657346664.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202312/a8iuOufB1703832570508.jpeg</t>
         </is>
       </c>
     </row>
@@ -5284,25 +5376,25 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>上海·SISP动漫游戏嘉年华</t>
+          <t>上海·《哈利的魔法世界》动漫视听音乐会</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>年家浜路518号 周浦万达广场</t>
+          <t>都市路4889号（莘庄地铁站南广场） 上海保利城市剧院</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2024.02.24 13:00-02.25 19:00</t>
+          <t>2024.02.24 14:30-02.24 16:00</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>111</v>
+        <v>5</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>158</t>
         </is>
       </c>
       <c r="H32" t="b">
@@ -5310,12 +5402,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80339</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80639</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202312/a8iuOufB1703832570508.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/dp013A4p1704783993628.png</t>
         </is>
       </c>
     </row>
@@ -5344,7 +5436,7 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2471</v>
+        <v>2486</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -5371,30 +5463,30 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2024-02-25</t>
+          <t>2024-02-24</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>上海·青山吉能见面会</t>
+          <t>上海·魔都元宵节漫展-COS为王</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>虹许路731号4号楼 THE BOXX•城市乐园</t>
+          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2024.02.25 14:30-02.25 19:30</t>
+          <t>2024.02.24 10:00-02.25 16:00</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>199</v>
+        <v>4</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>380</t>
+          <t>49</t>
         </is>
       </c>
       <c r="H34" t="b">
@@ -5402,12 +5494,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80142</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81238</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202312/1npuHFBM1703231674558.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/KxQZPADR1705913896609.jpeg</t>
         </is>
       </c>
     </row>
@@ -5417,30 +5509,30 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2024-03-02</t>
+          <t>2024-02-25</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>上海·原神X星穹铁道ONLY</t>
+          <t>上海·青山吉能见面会</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>逸仙路301号靠纪念路路口 上海宝丰联大酒店</t>
+          <t>虹许路731号4号楼 THE BOXX•城市乐园</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2024.03.02 10:00-03.02 17:00</t>
+          <t>2024.02.25 14:30-02.25 19:30</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>246</v>
+        <v>200</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>380</t>
         </is>
       </c>
       <c r="H35" t="b">
@@ -5448,12 +5540,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80299</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80142</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202312/V0xu26Cl1703753850690.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202312/1npuHFBM1703231674558.jpeg</t>
         </is>
       </c>
     </row>
@@ -5468,38 +5560,38 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>上海·小山百代2024上海粉丝见面会</t>
+          <t>上海·原神X星穹铁道ONLY</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>宜昌路179号 万代南梦宫上海文化中心</t>
+          <t>逸仙路301号靠纪念路路口 上海宝丰联大酒店</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2024.03.02 13:00-03.02 20:00</t>
+          <t>2024.03.02 10:00-03.02 17:00</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>226</v>
+        <v>252</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>380</t>
+          <t>60</t>
         </is>
       </c>
       <c r="H36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80924</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80299</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/FpA9OkKy1705467080070.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202312/V0xu26Cl1703753850690.jpeg</t>
         </is>
       </c>
     </row>
@@ -5509,43 +5601,43 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2024-03-03</t>
+          <t>2024-03-02</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>上海·怀旧番ONLY</t>
+          <t>上海·小山百代2024上海粉丝见面会</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>逸仙路270号  上海宝丰联大酒店</t>
+          <t>宜昌路179号 万代南梦宫上海文化中心</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2024.03.03 10:00-03.03 17:00</t>
+          <t>2024.03.02 13:00-03.02 20:00</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>124</v>
+        <v>235</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>380</t>
         </is>
       </c>
       <c r="H37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80575</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80924</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/y4uWdyPT1704700763902.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/FpA9OkKy1705467080070.jpeg</t>
         </is>
       </c>
     </row>
@@ -5555,30 +5647,30 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2024-03-09</t>
+          <t>2024-03-03</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>上海·S·CGE动漫游戏嘉年华</t>
+          <t>上海·怀旧番ONLY</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>军工路1076号 纪希片场(秀场)</t>
+          <t>逸仙路270号  上海宝丰联大酒店</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2024.03.09 10:00-03.10 17:00</t>
+          <t>2024.03.03 10:00-03.03 17:00</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>60</t>
         </is>
       </c>
       <c r="H38" t="b">
@@ -5586,12 +5678,12 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81173</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80575</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/TYA5FLkE1705891815532.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/y4uWdyPT1704700763902.jpeg</t>
         </is>
       </c>
     </row>
@@ -5606,38 +5698,38 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>上海·第五十三届燃梦星辰动漫嘉年华-随机宅舞</t>
+          <t>上海·S·CGE动漫游戏嘉年华</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>周家嘴路3608号 宝龙旭辉广场</t>
+          <t>军工路1076号 纪希片场(秀场)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2024.03.09 10:20-03.10 16:30</t>
+          <t>2024.03.09 10:00-03.10 17:00</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>70</t>
         </is>
       </c>
       <c r="H39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80571</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81173</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/SHH70VXN1704700240858.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/TYA5FLkE1705891815532.jpeg</t>
         </is>
       </c>
     </row>
@@ -5652,38 +5744,38 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>上海·青山刚昌ONLY【名侦探柯南&amp;魔术快斗】</t>
+          <t>上海·第五十三届燃梦星辰动漫嘉年华-随机宅舞</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>漕宝路1688号 诺宝中心酒店</t>
+          <t>周家嘴路3608号 宝龙旭辉广场</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2024.03.09 10:00-03.09 16:30</t>
+          <t>2024.03.09 10:20-03.10 16:30</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>865</v>
+        <v>43</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>58</t>
         </is>
       </c>
       <c r="H40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=76410</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80571</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202309/fVXMrcHy1693971682397.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/SHH70VXN1704700240858.jpeg</t>
         </is>
       </c>
     </row>
@@ -5693,30 +5785,30 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2024-03-16</t>
+          <t>2024-03-09</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>上海·三月的幻想演唱会2024「飞越蓝色时刻」</t>
+          <t>上海·青山刚昌ONLY【名侦探柯南&amp;魔术快斗】</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>宜昌路179号 万代南梦宫上海文化中心</t>
+          <t>漕宝路1688号 诺宝中心酒店</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2024.03.16 19:00-03.16 20:30</t>
+          <t>2024.03.09 10:00-03.09 16:30</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>40</v>
+        <v>875</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>380</t>
+          <t>73</t>
         </is>
       </c>
       <c r="H41" t="b">
@@ -5724,12 +5816,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80811</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=76410</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/TO6xpSqr1705289483473.png</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202309/fVXMrcHy1693971682397.jpeg</t>
         </is>
       </c>
     </row>
@@ -5744,25 +5836,25 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>上海·坏孩纸物语の第33届动漫节之庄子篇</t>
+          <t>上海·三月的幻想演唱会2024「飞越蓝色时刻」</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>中山北路3300号4楼L4001号 环球港上海世嘉都市乐园</t>
+          <t>宜昌路179号 万代南梦宫上海文化中心</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2024.03.16 10:00-03.17 21:00</t>
+          <t>2024.03.16 19:00-03.16 20:30</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>16</v>
+        <v>43</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>380</t>
         </is>
       </c>
       <c r="H42" t="b">
@@ -5770,12 +5862,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81138</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80811</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/jpr1lCt21705652306481.png</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/TO6xpSqr1705289483473.png</t>
         </is>
       </c>
     </row>
@@ -5785,30 +5877,30 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2024-03-30</t>
+          <t>2024-03-16</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>上海· TRUE（唐沢美帆）上海动漫交响音乐会</t>
+          <t>上海·坏孩纸物语の第33届动漫节之庄子篇</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>丁香路425号 上海东方艺术中心</t>
+          <t>中山北路3300号4楼L4001号 环球港上海世嘉都市乐园</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2024.03.30 19:30-03.30 21:00</t>
+          <t>2024.03.16 10:00-03.17 21:00</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>140</v>
+        <v>22</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>280</t>
+          <t>40</t>
         </is>
       </c>
       <c r="H43" t="b">
@@ -5816,12 +5908,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80906</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81138</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/FaJbLvS51705401178235.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/jpr1lCt21705652306481.png</t>
         </is>
       </c>
     </row>
@@ -5850,7 +5942,7 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -5877,30 +5969,30 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2024-04-05</t>
+          <t>2024-03-30</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>上海·第四届次元鹿角动漫游戏展</t>
+          <t>上海· TRUE（唐沢美帆）上海动漫交响音乐会</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>顾村镇蕰川路6号 智慧湾科创园</t>
+          <t>丁香路425号 上海东方艺术中心</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2024.04.05 10:00-04.06 17:00</t>
+          <t>2024.03.30 19:30-03.30 21:00</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>280</t>
         </is>
       </c>
       <c r="H45" t="b">
@@ -5908,12 +6000,12 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=78228</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80906</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202311/jgqIFxhx1699344723568.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/FaJbLvS51705401178235.jpeg</t>
         </is>
       </c>
     </row>
@@ -5923,43 +6015,43 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2024-04-06</t>
+          <t>2024-04-05</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>上海·从Butter-Fly到夏目之爱してる —— “好想大声说爱你”动漫钢琴演奏会</t>
+          <t>上海·第四届次元鹿角动漫游戏展</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>复兴中路1380号 捷豹上海交响音乐厅</t>
+          <t>顾村镇蕰川路6号 智慧湾科创园</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2024.04.06 19:30-04.06 21:30</t>
+          <t>2024.04.05 10:00-04.06 17:00</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>60</t>
         </is>
       </c>
       <c r="H46" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80050</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=78228</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202312/0iJP3TY61703056498448.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202311/jgqIFxhx1699344723568.jpeg</t>
         </is>
       </c>
     </row>
@@ -5969,26 +6061,26 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2024-04-13</t>
+          <t>2024-04-06</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>上海·《四月是你的谎言》——“公生”与“薰”的钢琴小提琴唯美经典音乐集</t>
+          <t>上海·从Butter-Fly到夏目之爱してる —— “好想大声说爱你”动漫钢琴演奏会</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>丁香路425号 上海东方艺术中心</t>
+          <t>复兴中路1380号 捷豹上海交响音乐厅</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2024.04.13 19:30-04.13 21:30</t>
+          <t>2024.04.06 19:30-04.06 21:30</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>171</v>
+        <v>10</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -6000,12 +6092,12 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=78667</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80050</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202311/bTP7w6GD1700130122940.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202312/0iJP3TY61703056498448.jpeg</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6126,7 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -6080,7 +6172,7 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -6126,7 +6218,7 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -6172,7 +6264,7 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update gh-pages to output generated at 0b82ce7
</commit_message>
<xml_diff>
--- a/上海-漫展信息.xlsx
+++ b/上海-漫展信息.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,38 +482,38 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2023-11-02</t>
+          <t>2023-12-10</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>上海·Hello Kitty Cosmos 50周年光影特展</t>
+          <t>上海·多维跃迁-2023 红点设计概念大奖获奖作品展</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>漕宝路3055号 宝龙美术馆</t>
+          <t>国展路1099号 上海世博展览馆</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2023.11.02 10:00-2024.01.28 18:00</t>
+          <t>2023.12.10 12:00-2024.02.16 17:00</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>124</v>
+        <v>34</v>
       </c>
       <c r="G2" t="n">
-        <v>139</v>
+        <v>80</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=77862</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=78809</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202310/QnmD4yOd1698652192047.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202311/YsBoZAOW1700551290654.jpeg</t>
         </is>
       </c>
     </row>
@@ -523,38 +523,38 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2023-12-10</t>
+          <t>2023-12-22</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>上海·多维跃迁-2023 红点设计概念大奖获奖作品展</t>
+          <t>上海·新海诚导演作品《铃芽之旅》展 丨 购票抽新海诚见面会门票丨 超限定复刻原画发售</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>国展路1099号 上海世博展览馆</t>
+          <t>湖滨路168号 上海无限极荟购物中心</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2023.12.10 12:00-2024.02.16 17:00</t>
+          <t>2023.12.22 10:00-2024.02.16 22:00</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>34</v>
+        <v>1696</v>
       </c>
       <c r="G3" t="n">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=78809</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=79166</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202311/YsBoZAOW1700551290654.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202311/MjTiIYlk1701242361853.jpeg</t>
         </is>
       </c>
     </row>
@@ -564,38 +564,38 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2023-12-22</t>
+          <t>2024-01-27</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>上海·新海诚导演作品《铃芽之旅》展 丨 购票抽新海诚见面会门票丨 超限定复刻原画发售</t>
+          <t>上海·第八届次元鹿角动漫游戏展</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>湖滨路168号 上海无限极荟购物中心</t>
+          <t>吴中路1588号上海爱琴海购物中心F4 竞梦元宇宙</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2023.12.22 10:00-2024.02.16 22:00</t>
+          <t>2024.01.27 10:00-01.28 21:00</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1694</v>
+        <v>1239</v>
       </c>
       <c r="G4" t="n">
-        <v>55</v>
+        <v>98</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79166</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80979</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202311/MjTiIYlk1701242361853.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/xPOF923U1705545223366.jpeg</t>
         </is>
       </c>
     </row>
@@ -605,38 +605,38 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2024-01-27</t>
+          <t>2024-01-31</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>上海·同好召集令火影only</t>
+          <t>上海·寻迹冬日LOVELIVE同好会</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>市真南路1199弄1号 智创TOP综合体产城</t>
+          <t>愚园路1250号 新歌空间</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2024.01.27 10:00-01.28 18:00</t>
+          <t>2024.01.31 11:30-01.31 17:00</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>575</v>
+        <v>194</v>
       </c>
       <c r="G5" t="n">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80284</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=79332</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/9xGb6MXN1704183627126.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202312/Ewreg1JT1701677993728.jpeg</t>
         </is>
       </c>
     </row>
@@ -646,38 +646,38 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2024-01-27</t>
+          <t>2024-02-03</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>上海·第八届次元鹿角动漫游戏展</t>
+          <t>上海·Coser迎春动漫展</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>吴中路1588号上海爱琴海购物中心F4 竞梦元宇宙</t>
+          <t>海潮路133号B1 JUMP工坊</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2024.01.27 10:00-01.28 21:00</t>
+          <t>2024.02.03 10:00-02.04 17:00</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1237</v>
+        <v>912</v>
       </c>
       <c r="G6" t="n">
-        <v>98</v>
+        <v>60</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80979</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80646</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/xPOF923U1705545223366.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/4WVkFc4d1704787729064.jpeg</t>
         </is>
       </c>
     </row>
@@ -687,38 +687,38 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2024-01-27</t>
+          <t>2024-02-03</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>上海·魔都寒假漫展-CF01</t>
+          <t>上海·ENP电次元派对vol.04</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
+          <t>人民大道221号 迪美购物中心</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2024.01.27 10:00-01.28 16:00</t>
+          <t>2024.02.03 18:30-02.03 22:00</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1020</v>
+        <v>24</v>
       </c>
       <c r="G7" t="n">
-        <v>59</v>
+        <v>99</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80204</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80945</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202312/eK96fdcg1703573110264.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/1sjalWS51705479361512.jpeg</t>
         </is>
       </c>
     </row>
@@ -728,38 +728,38 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2024-01-28</t>
+          <t>2024-02-03</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>上海 ·WOW潮元原神x星铁主题二次元狂欢派对</t>
+          <t>上海·偶像梦幻祭红白歌合战Only</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>政通路189号五角场万达广场C栋 元气森林livehouse</t>
+          <t>虹许路731号4号楼 THE BOXX•城市乐园</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2024.01.28 14:00-01.28 19:00</t>
+          <t>2024.02.03 13:30-02.03 22:00</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>456</v>
+        <v>105</v>
       </c>
       <c r="G8" t="n">
-        <v>149</v>
+        <v>88</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80167</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81199</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/QTp32HEM1705028548091.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/C7E7svbZ1705903245860.jpeg</t>
         </is>
       </c>
     </row>
@@ -769,40 +769,38 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2024-01-28</t>
+          <t>2024-02-03</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>上海·Comic World动漫游园会（取消）</t>
+          <t>上海·第七届次元鹿角二次元派对</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>盈浦街道淀山浦社区淀山湖大道851号青浦万达茂F3 万达汽车乐园(青浦万达茂店)</t>
+          <t>长宁路1191号来福士西区(W)B1层01号、11号 星零界</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2024.01.28 09:30-01.28 17:00</t>
+          <t>2024.02.03 10:00-02.04 17:00</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2218</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>不可售</t>
-        </is>
+        <v>1346</v>
+      </c>
+      <c r="G9" t="n">
+        <v>98</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=78523</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=79938</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/HAkxl2611705480975408.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/b1XT2w4T1705027781100.jpeg</t>
         </is>
       </c>
     </row>
@@ -812,38 +810,38 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2024-01-28</t>
+          <t>2024-02-10</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>上海·坏孩纸物语の第32届动漫节之冬日季</t>
+          <t>上海·寒假CF漫展-春节档-神龙在世</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>剑川路1000号 闵行龙湖天街</t>
+          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2024.01.28 14:00-01.28 20:00</t>
+          <t>2024.02.10 10:00-02.17 16:00</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>746</v>
+        <v>44</v>
       </c>
       <c r="G10" t="n">
-        <v>36.9</v>
+        <v>49</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80871</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81192</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/5fmQrQJ81705573963752.png</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/S8XxkA631705896741998.jpeg</t>
         </is>
       </c>
     </row>
@@ -853,38 +851,38 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2024-01-28</t>
+          <t>2024-02-14</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>上海·次元裂缝-X 新年二次元偶像日</t>
+          <t>上海·原X铁X崩only</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>海潮路133号B1 JUMP工坊</t>
+          <t>澳门路168号 月星国际家居</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2024.01.28 14:00-01.28 18:00</t>
+          <t>2024.02.14 10:30-02.14 16:30</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>90</v>
+        <v>43</v>
       </c>
       <c r="G11" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80999</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81446</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/lNroHqJY1705549448993.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/IIePRulM1706248855263.jpeg</t>
         </is>
       </c>
     </row>
@@ -894,38 +892,38 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2024-01-31</t>
+          <t>2024-02-14</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>上海·寻迹冬日LOVELIVE同好会</t>
+          <t>上海·奇卡波利动漫嘉年华</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>愚园路1250号 新歌空间</t>
+          <t>申滨路36号 虹桥丽宝广场</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2024.01.31 11:30-01.31 17:00</t>
+          <t>2024.02.14 10:00-02.14 17:00</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>194</v>
+        <v>77</v>
       </c>
       <c r="G12" t="n">
-        <v>83</v>
+        <v>48.8</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79332</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81260</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202312/Ewreg1JT1701677993728.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/9OHovK2V1705978109130.jpeg</t>
         </is>
       </c>
     </row>
@@ -935,38 +933,38 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2024-02-03</t>
+          <t>2024-02-14</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>上海·Coser迎春动漫展</t>
+          <t>上海·魔都COS漫展-情人节专场AM01</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>海潮路133号B1 JUMP工坊</t>
+          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2024.02.03 10:00-02.04 17:00</t>
+          <t>2024.02.14 10:00-02.14 16:00</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>858</v>
+        <v>106</v>
       </c>
       <c r="G13" t="n">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80646</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80691</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/4WVkFc4d1704787729064.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/aSdjV6Kw1704868345679.jpeg</t>
         </is>
       </c>
     </row>
@@ -976,38 +974,38 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2024-02-03</t>
+          <t>2024-02-16</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>上海·ENP电次元派对vol.04</t>
+          <t>上海·次元裂缝-X 新年anikura派对</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>人民大道221号 迪美购物中心</t>
+          <t>海潮路133号B1 JUMP工坊</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2024.02.03 18:30-02.03 22:00</t>
+          <t>2024.02.16 14:00-02.16 19:00</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="G14" t="n">
-        <v>99</v>
+        <v>60</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80945</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81314</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/1sjalWS51705479361512.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/OrhHWKdR1706062360956.jpeg</t>
         </is>
       </c>
     </row>
@@ -1017,38 +1015,38 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2024-02-03</t>
+          <t>2024-02-16</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>上海·偶像梦幻祭红白歌合战Only</t>
+          <t>上海·第九届次元鹿角动漫游戏展</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>虹许路731号4号楼 THE BOXX•城市乐园</t>
+          <t>盈浦街道淀山浦社区淀山湖大道851号青浦万达茂F3 万达汽车乐园(青浦万达茂店)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2024.02.03 13:30-02.03 22:00</t>
+          <t>2024.02.16 11:00-02.17 18:00</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>93</v>
+        <v>1264</v>
       </c>
       <c r="G15" t="n">
-        <v>88</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81199</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80497</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/C7E7svbZ1705903245860.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/0duSXTQy1704423309244.jpeg</t>
         </is>
       </c>
     </row>
@@ -1058,38 +1056,38 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2024-02-03</t>
+          <t>2024-02-17</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>上海·第七届次元鹿角二次元派对</t>
+          <t>上海·少女番only2.0</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>长宁路1191号来福士西区(W)B1层01号、11号 星零界</t>
+          <t>营口路699号(黄兴公园地铁站2号口旁) 花嫁丽舍</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2024.02.03 10:00-02.04 17:00</t>
+          <t>2024.02.17 10:00-02.17 17:00</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>1331</v>
+        <v>364</v>
       </c>
       <c r="G16" t="n">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79938</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81148</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/b1XT2w4T1705027781100.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/j6eEZ18S1705657346664.jpeg</t>
         </is>
       </c>
     </row>
@@ -1099,38 +1097,38 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2024-02-10</t>
+          <t>2024-02-24</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>上海·寒假CF漫展-春节档-神龙在世</t>
+          <t>上海·SISPmini动漫游戏嘉年华</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
+          <t>剑川路1000号 龙湖上海闵行天街</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2024.02.10 10:00-02.17 16:00</t>
+          <t>2024.02.24 13:00-02.25 19:00</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>38</v>
+        <v>434</v>
       </c>
       <c r="G17" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81192</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=79046</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/S8XxkA631705896741998.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/jzovdppq1706166165502.jpeg</t>
         </is>
       </c>
     </row>
@@ -1140,38 +1138,38 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2024-02-14</t>
+          <t>2024-02-24</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>上海·原X铁X崩only</t>
+          <t>上海·SISP动漫游戏嘉年华</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>澳门路168号 月星国际家居</t>
+          <t>年家浜路518号 周浦万达广场</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2024.02.14 10:30-02.14 16:30</t>
+          <t>2024.02.24 13:00-02.25 19:00</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>28</v>
+        <v>121</v>
       </c>
       <c r="G18" t="n">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81446</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80339</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/IIePRulM1706248855263.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202312/a8iuOufB1703832570508.jpeg</t>
         </is>
       </c>
     </row>
@@ -1181,38 +1179,38 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2024-02-14</t>
+          <t>2024-02-24</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>上海·奇卡波利动漫嘉年华</t>
+          <t>上海·原神×崩坏×星铁only旅行盛宴2.0</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>申滨路36号 虹桥丽宝广场</t>
+          <t>西藏南路1号 上海大世界</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2024.02.14 10:00-02.14 17:00</t>
+          <t>2024.02.24 10:00-02.25 17:00</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>67</v>
+        <v>133</v>
       </c>
       <c r="G19" t="n">
-        <v>48.8</v>
+        <v>65</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81260</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81276</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/9OHovK2V1705978109130.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/82hU3z8m1706155835021.png</t>
         </is>
       </c>
     </row>
@@ -1222,38 +1220,38 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2024-02-14</t>
+          <t>2024-02-24</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>上海·魔都COS漫展-情人节专场AM01</t>
+          <t>上海·第三届燃梦BACG PRO游戏动漫展-原X铁X崩同好交流</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
+          <t>盈浦街道淀山浦社区淀山湖大道851号青浦万达茂F3 万达汽车乐园(青浦万达茂店)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2024.02.14 10:00-02.14 16:00</t>
+          <t>2024.02.24 11:00-02.25 16:30</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>101</v>
+        <v>2514</v>
       </c>
       <c r="G20" t="n">
-        <v>49</v>
+        <v>65.8</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80691</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=77754</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/aSdjV6Kw1704868345679.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202312/7eGZETK91701943985671.jpeg</t>
         </is>
       </c>
     </row>
@@ -1263,38 +1261,38 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2024-02-16</t>
+          <t>2024-02-24</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>上海·次元裂缝-X 新年anikura派对</t>
+          <t>上海·趣元界&amp;斗罗大陆上元佳节次元派对</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>海潮路133号B1 JUMP工坊</t>
+          <t>长宁路1191号长宁来福士B1 长宁来福士</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2024.02.16 14:00-02.16 19:00</t>
+          <t>2024.02.24 11:30-02.25 17:30</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>31</v>
+        <v>511</v>
       </c>
       <c r="G21" t="n">
-        <v>60</v>
+        <v>98</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81314</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81415</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/OrhHWKdR1706062360956.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/yis4JHfE1706169986733.jpeg</t>
         </is>
       </c>
     </row>
@@ -1304,38 +1302,38 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2024-02-16</t>
+          <t>2024-02-24</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>上海·第九届次元鹿角动漫游戏展</t>
+          <t>上海·魔都元宵节漫展-COS为王</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>盈浦街道淀山浦社区淀山湖大道851号青浦万达茂F3 万达汽车乐园(青浦万达茂店)</t>
+          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2024.02.16 11:00-02.17 18:00</t>
+          <t>2024.02.24 10:00-02.25 16:00</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>1251</v>
+        <v>11</v>
       </c>
       <c r="G22" t="n">
-        <v>65.90000000000001</v>
+        <v>49</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80497</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81238</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/0duSXTQy1704423309244.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/KxQZPADR1705913896609.jpeg</t>
         </is>
       </c>
     </row>
@@ -1345,38 +1343,38 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2024-02-17</t>
+          <t>2024-02-24</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>上海·少女番only2.0</t>
+          <t>上海·魔都多厨狂喜漫展-CH01</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>营口路699号(黄兴公园地铁站2号口旁) 花嫁丽舍</t>
+          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2024.02.17 10:00-02.17 17:00</t>
+          <t>2024.02.24 10:00-02.25 16:00</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>351</v>
+        <v>3</v>
       </c>
       <c r="G23" t="n">
-        <v>80</v>
+        <v>49</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81148</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81423</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/j6eEZ18S1705657346664.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/axpOY3zo1706173660010.jpeg</t>
         </is>
       </c>
     </row>
@@ -1386,38 +1384,38 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2024-02-24</t>
+          <t>2024-03-02</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>上海·SISPmini动漫游戏嘉年华</t>
+          <t>上海·原神X星穹铁道ONLY</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>剑川路1000号 龙湖上海闵行天街</t>
+          <t>逸仙路301号靠纪念路路口 上海宝丰联大酒店</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2024.02.24 13:00-02.25 19:00</t>
+          <t>2024.03.02 10:00-03.02 17:00</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>426</v>
+        <v>264</v>
       </c>
       <c r="G24" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79046</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80299</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/jzovdppq1706166165502.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202312/V0xu26Cl1703753850690.jpeg</t>
         </is>
       </c>
     </row>
@@ -1427,38 +1425,38 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2024-02-24</t>
+          <t>2024-03-03</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>上海·SISP动漫游戏嘉年华</t>
+          <t>上海·怀旧番ONLY</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>年家浜路518号 周浦万达广场</t>
+          <t>逸仙路270号  上海宝丰联大酒店</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2024.02.24 13:00-02.25 19:00</t>
+          <t>2024.03.03 10:00-03.03 17:00</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>119</v>
+        <v>155</v>
       </c>
       <c r="G25" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80339</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80575</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202312/a8iuOufB1703832570508.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/y4uWdyPT1704700763902.jpeg</t>
         </is>
       </c>
     </row>
@@ -1468,38 +1466,38 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2024-02-24</t>
+          <t>2024-03-08</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>上海·原神×崩坏×星铁only旅行盛宴2.0</t>
+          <t>上海·第八届ACBC动漫盛典-国潮汉服游园会</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>西藏南路1号 上海大世界</t>
+          <t>浦锦南路1586弄2号 奇迹花园</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2024.02.24 10:00-02.25 17:00</t>
+          <t>2024.03.08 10:00-03.10 17:00</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>119</v>
+        <v>5</v>
       </c>
       <c r="G26" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81276</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81456</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/82hU3z8m1706155835021.png</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/qZtpawf51706254849667.jpeg</t>
         </is>
       </c>
     </row>
@@ -1509,38 +1507,38 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2024-02-24</t>
+          <t>2024-03-09</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>上海·第三届燃梦BACG PRO游戏动漫展-原X铁X崩同好交流</t>
+          <t>上海·S·CGE动漫游戏嘉年华</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>盈浦街道淀山浦社区淀山湖大道851号青浦万达茂F3 万达汽车乐园(青浦万达茂店)</t>
+          <t>军工路1076号 纪希片场(秀场)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2024.02.24 11:00-02.25 16:30</t>
+          <t>2024.03.09 10:00-03.10 17:00</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2511</v>
+        <v>73</v>
       </c>
       <c r="G27" t="n">
-        <v>65.8</v>
+        <v>70</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=77754</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81173</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202312/7eGZETK91701943985671.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/TYA5FLkE1705891815532.jpeg</t>
         </is>
       </c>
     </row>
@@ -1550,38 +1548,38 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2024-02-24</t>
+          <t>2024-03-09</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>上海·趣元界&amp;斗罗大陆上元佳节次元派对</t>
+          <t>上海·第五十三届燃梦星辰动漫嘉年华-随机宅舞</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>长宁路1191号长宁来福士B1 长宁来福士</t>
+          <t>周家嘴路3608号 宝龙旭辉广场</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2024.02.24 11:30-02.25 17:30</t>
+          <t>2024.03.09 10:20-03.10 16:30</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>509</v>
+        <v>49</v>
       </c>
       <c r="G28" t="n">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81415</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80571</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/yis4JHfE1706169986733.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/SHH70VXN1704700240858.jpeg</t>
         </is>
       </c>
     </row>
@@ -1591,38 +1589,38 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2024-02-24</t>
+          <t>2024-03-09</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>上海·魔都元宵节漫展-COS为王</t>
+          <t>上海·青山刚昌ONLY【名侦探柯南&amp;魔术快斗】</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
+          <t>漕宝路1688号 诺宝中心酒店</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2024.02.24 10:00-02.25 16:00</t>
+          <t>2024.03.09 10:00-03.09 16:30</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>11</v>
+        <v>896</v>
       </c>
       <c r="G29" t="n">
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81238</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=76410</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/KxQZPADR1705913896609.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202309/fVXMrcHy1693971682397.jpeg</t>
         </is>
       </c>
     </row>
@@ -1632,38 +1630,38 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2024-02-24</t>
+          <t>2024-03-16</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>上海·魔都多厨狂喜漫展-CH01</t>
+          <t>上海·坏孩纸物语の第33届动漫节之庄子篇</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
+          <t>中山北路3300号4楼L4001号 环球港上海世嘉都市乐园</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2024.02.24 10:00-02.25 16:00</t>
+          <t>2024.03.16 10:00-03.17 21:00</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="G30" t="n">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81423</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81138</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/axpOY3zo1706173660010.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/jpr1lCt21705652306481.png</t>
         </is>
       </c>
     </row>
@@ -1673,38 +1671,38 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2024-03-02</t>
+          <t>2024-04-05</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>上海·原神X星穹铁道ONLY</t>
+          <t>上海·第四届次元鹿角动漫游戏展</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>逸仙路301号靠纪念路路口 上海宝丰联大酒店</t>
+          <t>顾村镇蕰川路6号 智慧湾科创园</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2024.03.02 10:00-03.02 17:00</t>
+          <t>2024.04.05 10:00-04.06 17:00</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>260</v>
+        <v>63</v>
       </c>
       <c r="G31" t="n">
         <v>60</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80299</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=78228</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202312/V0xu26Cl1703753850690.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202311/jgqIFxhx1699344723568.jpeg</t>
         </is>
       </c>
     </row>
@@ -1714,38 +1712,38 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2024-03-03</t>
+          <t>2024-04-27</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>上海·怀旧番ONLY</t>
+          <t>上海·  第五十三届妖漫动漫游戏展</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>逸仙路270号  上海宝丰联大酒店</t>
+          <t>曹杨路1888号 复悦荟</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2024.03.03 10:00-03.03 17:00</t>
+          <t>2024.04.27 10:00-04.27 17:00</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="G32" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80575</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=78657</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/y4uWdyPT1704700763902.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/tamNdgEN1705331335847.jpeg</t>
         </is>
       </c>
     </row>
@@ -1755,38 +1753,38 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2024-03-08</t>
+          <t>2024-05-01</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>上海·第八届ACBC动漫盛典-国潮汉服游园会</t>
+          <t>上海·S·CGE动漫游戏嘉年华</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>浦锦南路1586弄2号 奇迹花园</t>
+          <t>军工路1076号 纪希片场(秀场)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2024.03.08 10:00-03.10 17:00</t>
+          <t>2024.05.01 10:00-05.02 17:00</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="G33" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81456</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81204</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/qZtpawf51706254849667.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/nbFRULYe1705904589212.jpeg</t>
         </is>
       </c>
     </row>
@@ -1796,38 +1794,38 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2024-03-09</t>
+          <t>2024-05-01</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>上海·S·CGE动漫游戏嘉年华</t>
+          <t>上海·魔都野良神only</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>军工路1076号 纪希片场(秀场)</t>
+          <t>南京东路830号 第一百货</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2024.03.09 10:00-03.10 17:00</t>
+          <t>2024.05.01 10:00-05.01 17:00</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>62</v>
+        <v>215</v>
       </c>
       <c r="G34" t="n">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81173</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80321</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/TYA5FLkE1705891815532.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/KBlb0enU1704358750268.jpeg</t>
         </is>
       </c>
     </row>
@@ -1837,323 +1835,36 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2024-03-09</t>
+          <t>2024-05-05</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>上海·第五十三届燃梦星辰动漫嘉年华-随机宅舞</t>
+          <t>上海·灌篮高手--青春永不散场</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>周家嘴路3608号 宝龙旭辉广场</t>
+          <t>逸仙路1328弄 新业坊</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2024.03.09 10:20-03.10 16:30</t>
+          <t>2024.05.05 10:00-05.05 17:00</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="G35" t="n">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80571</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80835</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
-        <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/SHH70VXN1704700240858.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="1" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>2024-03-09</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>上海·青山刚昌ONLY【名侦探柯南&amp;魔术快斗】</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>漕宝路1688号 诺宝中心酒店</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>2024.03.09 10:00-03.09 16:30</t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>893</v>
-      </c>
-      <c r="G36" t="n">
-        <v>73</v>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=76410</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202309/fVXMrcHy1693971682397.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="1" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>2024-03-16</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>上海·坏孩纸物语の第33届动漫节之庄子篇</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>中山北路3300号4楼L4001号 环球港上海世嘉都市乐园</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>2024.03.16 10:00-03.17 21:00</t>
-        </is>
-      </c>
-      <c r="F37" t="n">
-        <v>29</v>
-      </c>
-      <c r="G37" t="n">
-        <v>40</v>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81138</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/jpr1lCt21705652306481.png</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="1" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>2024-04-05</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>上海·第四届次元鹿角动漫游戏展</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>顾村镇蕰川路6号 智慧湾科创园</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>2024.04.05 10:00-04.06 17:00</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>63</v>
-      </c>
-      <c r="G38" t="n">
-        <v>60</v>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=78228</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202311/jgqIFxhx1699344723568.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="1" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>2024-04-27</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>上海·  第五十三届妖漫动漫游戏展</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>曹杨路1888号 复悦荟</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>2024.04.27 10:00-04.27 17:00</t>
-        </is>
-      </c>
-      <c r="F39" t="n">
-        <v>149</v>
-      </c>
-      <c r="G39" t="n">
-        <v>80</v>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=78657</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/tamNdgEN1705331335847.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="1" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>2024-05-01</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>上海·S·CGE动漫游戏嘉年华</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>军工路1076号 纪希片场(秀场)</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>2024.05.01 10:00-05.02 17:00</t>
-        </is>
-      </c>
-      <c r="F40" t="n">
-        <v>17</v>
-      </c>
-      <c r="G40" t="n">
-        <v>70</v>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81204</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/nbFRULYe1705904589212.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="1" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>2024-05-01</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>上海·魔都野良神only</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>南京东路830号 第一百货</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>2024.05.01 10:00-05.01 17:00</t>
-        </is>
-      </c>
-      <c r="F41" t="n">
-        <v>209</v>
-      </c>
-      <c r="G41" t="n">
-        <v>79</v>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80321</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/KBlb0enU1704358750268.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="1" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>2024-05-05</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>上海·灌篮高手--青春永不散场</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>逸仙路1328弄 新业坊</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>2024.05.05 10:00-05.05 17:00</t>
-        </is>
-      </c>
-      <c r="F42" t="n">
-        <v>16</v>
-      </c>
-      <c r="G42" t="n">
-        <v>89</v>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80835</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
         <is>
           <t>//i1.hdslb.com/bfs/openplatform/202401/hdaVclFC1705301931054.jpeg</t>
         </is>
@@ -2170,7 +1881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2284,7 +1995,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G3" t="n">
         <v>90</v>
@@ -2306,40 +2017,38 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2024-01-01</t>
+          <t>2024-02-02</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>上海·沉浸式悬念剧场《9号秘事》</t>
+          <t>上海·次元LAB 二次元电音节</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>人民大道300号 上海大剧院</t>
+          <t>中兴路1683号金融街购物中心L3-27 蜚声上海Livehouse</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2024.01.01 19:30-01.28 16:20</t>
+          <t>2024.02.02 12:30-02.02 21:00</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>不可售</t>
-        </is>
+        <v>682</v>
+      </c>
+      <c r="G4" t="n">
+        <v>380</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79939</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80128</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202312/hY6FVnjM1702954652593.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202312/DEW1XYty1703226993965.jpeg</t>
         </is>
       </c>
     </row>
@@ -2349,38 +2058,38 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2024-02-02</t>
+          <t>2024-02-04</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>上海·次元LAB 二次元电音节</t>
+          <t>上海·触手猴钢琴巡演·marasy piano live tour『生音』上海站·Powered by 东方弹幕神乐失落幻想</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>中兴路1683号金融街购物中心L3-27 蜚声上海Livehouse</t>
+          <t>丁香路425号(上海科技馆地铁站1号口步行460米) 上海东方艺术中心音乐厅</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2024.02.02 12:30-02.02 21:00</t>
+          <t>2024.02.04 19:30-02.04 21:00</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>673</v>
+        <v>516</v>
       </c>
       <c r="G5" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80128</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80734</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202312/DEW1XYty1703226993965.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/IcjPp0TE1704951328918.jpeg</t>
         </is>
       </c>
     </row>
@@ -2390,38 +2099,38 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2024-02-04</t>
+          <t>2024-02-14</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>上海·触手猴钢琴巡演·marasy piano live tour『生音』上海站·Powered by 东方弹幕神乐失落幻想</t>
+          <t>上海·【情人节特辑】《那年我们》记忆重启韩剧经典OST音乐会《请回答1988》《来自星星的你》</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>丁香路425号(上海科技馆地铁站1号口步行460米) 上海东方艺术中心音乐厅</t>
+          <t>牛庄路704号 中国大戏院</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2024.02.04 19:30-02.04 21:00</t>
+          <t>2024.02.14 19:30-02.14 21:00</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>475</v>
+        <v>6</v>
       </c>
       <c r="G6" t="n">
-        <v>280</v>
+        <v>80</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80734</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80615</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/IcjPp0TE1704951328918.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/5DDVhKcO1704767761361.png</t>
         </is>
       </c>
     </row>
@@ -2431,38 +2140,38 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2024-02-14</t>
+          <t>2024-02-24</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>上海·【情人节特辑】《那年我们》记忆重启韩剧经典OST音乐会《请回答1988》《来自星星的你》</t>
+          <t>上海·《哈利的魔法世界》动漫视听音乐会</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>牛庄路704号 中国大戏院</t>
+          <t>都市路4889号（莘庄地铁站南广场） 上海保利城市剧院</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2024.02.14 19:30-02.14 21:00</t>
+          <t>2024.02.24 14:30-02.24 16:00</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G7" t="n">
-        <v>80</v>
+        <v>158</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80615</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80639</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/5DDVhKcO1704767761361.png</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/4PieCC9N1706261750579.jpeg</t>
         </is>
       </c>
     </row>
@@ -2472,38 +2181,38 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2024-02-24</t>
+          <t>2024-02-25</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>上海·《哈利的魔法世界》动漫视听音乐会</t>
+          <t>上海·青山吉能见面会</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>都市路4889号（莘庄地铁站南广场） 上海保利城市剧院</t>
+          <t>虹许路731号4号楼 THE BOXX•城市乐园</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2024.02.24 14:30-02.24 16:00</t>
+          <t>2024.02.25 14:30-02.25 19:30</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>9</v>
+        <v>207</v>
       </c>
       <c r="G8" t="n">
-        <v>158</v>
+        <v>380</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80639</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80142</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/4PieCC9N1706261750579.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202312/1npuHFBM1703231674558.jpeg</t>
         </is>
       </c>
     </row>
@@ -2513,38 +2222,38 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2024-02-25</t>
+          <t>2024-03-02</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>上海·青山吉能见面会</t>
+          <t>上海·2024藤田玲上海粉丝见面会</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>虹许路731号4号楼 THE BOXX•城市乐园</t>
+          <t>宜昌路179号 万代南梦宫上海文化中心</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2024.02.25 14:30-02.25 19:30</t>
+          <t>2024.03.02 12:30-03.02 19:40</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>205</v>
+        <v>11</v>
       </c>
       <c r="G9" t="n">
-        <v>380</v>
+        <v>580</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80142</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80993</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202312/1npuHFBM1703231674558.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/Vm6ntgVd1705548188785.png</t>
         </is>
       </c>
     </row>
@@ -2559,7 +2268,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>上海·2024藤田玲上海粉丝见面会</t>
+          <t>上海·小山百代2024上海粉丝见面会</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2569,23 +2278,23 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2024.03.02 12:30-03.02 19:40</t>
+          <t>2024.03.02 13:00-03.02 20:00</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>9</v>
+        <v>253</v>
       </c>
       <c r="G10" t="n">
-        <v>580</v>
+        <v>380</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80993</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80924</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/Vm6ntgVd1705548188785.png</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/FpA9OkKy1705467080070.jpeg</t>
         </is>
       </c>
     </row>
@@ -2595,38 +2304,38 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2024-03-02</t>
+          <t>2024-03-09</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>上海·小山百代2024上海粉丝见面会</t>
+          <t>上海·《挪威的森林》—摇滚情歌之夜演唱会</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>宜昌路179号 万代南梦宫上海文化中心</t>
+          <t>南京西路1376号 上海商城剧院</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2024.03.02 13:00-03.02 20:00</t>
+          <t>2024.03.09 19:30-03.09 21:00</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>249</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>380</v>
+        <v>72</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80924</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81241</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/FpA9OkKy1705467080070.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/1FJ0Fj5m1705915336335.jpeg</t>
         </is>
       </c>
     </row>
@@ -2641,7 +2350,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>上海·《挪威的森林》—摇滚情歌之夜演唱会</t>
+          <t>上海·爱乐之城音乐会</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2651,23 +2360,23 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2024.03.09 19:30-03.09 21:00</t>
+          <t>2024.03.09 14:00-03.09 15:30</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G12" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81241</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81289</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/1FJ0Fj5m1705915336335.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/ZZXtDrwZ1705996679699.jpeg</t>
         </is>
       </c>
     </row>
@@ -2677,38 +2386,38 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2024-03-09</t>
+          <t>2024-03-16</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>上海·爱乐之城音乐会</t>
+          <t>上海·三月的幻想演唱会2024「飞越蓝色时刻」</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>南京西路1376号 上海商城剧院</t>
+          <t>宜昌路179号 万代南梦宫上海文化中心</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2024.03.09 14:00-03.09 15:30</t>
+          <t>2024.03.16 19:00-03.16 20:30</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2</v>
+        <v>52</v>
       </c>
       <c r="G13" t="n">
-        <v>60</v>
+        <v>380</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81289</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80811</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/ZZXtDrwZ1705996679699.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/TO6xpSqr1705289483473.png</t>
         </is>
       </c>
     </row>
@@ -2718,38 +2427,38 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2024-03-16</t>
+          <t>2024-03-17</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>上海·三月的幻想演唱会2024「飞越蓝色时刻」</t>
+          <t>上海 ·《疯狂动物城》动漫视听音乐会</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>宜昌路179号 万代南梦宫上海文化中心</t>
+          <t>牛庄路704号 中国大戏院</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2024.03.16 19:00-03.16 20:30</t>
+          <t>2024.03.17 15:30-03.17 17:00</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="G14" t="n">
-        <v>380</v>
+        <v>80</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80811</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81112</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/TO6xpSqr1705289483473.png</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/Wg8b6SRn1705651166088.png</t>
         </is>
       </c>
     </row>
@@ -2764,33 +2473,33 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>上海 ·《疯狂动物城》动漫视听音乐会</t>
+          <t>上海·amazarashi Asia Tour 2024 「永遠市 -Eternal City-」上海公演</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>牛庄路704号 中国大戏院</t>
+          <t>宜昌路179号 万代南梦宫上海文化中心</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2024.03.17 15:30-03.17 17:00</t>
+          <t>2024.03.17 18:00-03.17 19:30</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>5</v>
+        <v>686</v>
       </c>
       <c r="G15" t="n">
-        <v>80</v>
+        <v>480</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81112</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81039</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/Wg8b6SRn1705651166088.png</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/icsawZU11705566039011.jpeg</t>
         </is>
       </c>
     </row>
@@ -2805,33 +2514,33 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>上海·amazarashi Asia Tour 2024 「永遠市 -Eternal City-」上海公演</t>
+          <t>上海·《笑傲江湖》经典武侠影视金曲音乐会</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>宜昌路179号 万代南梦宫上海文化中心</t>
+          <t>牛庄路704号 中国大戏院</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2024.03.17 18:00-03.17 19:30</t>
+          <t>2024.03.17 19:30-03.17 21:00</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>643</v>
+        <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>480</v>
+        <v>80</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81039</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80875</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/icsawZU11705566039011.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/8AwIAy4I1705385447242.jpeg</t>
         </is>
       </c>
     </row>
@@ -2846,33 +2555,33 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>上海·《笑傲江湖》经典武侠影视金曲音乐会</t>
+          <t>上海·遇见新海诚--帝玖「这次一定」室内乐ACG音乐会</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>牛庄路704号 中国大戏院</t>
+          <t>延安东路523号 凯迪拉克·上海音乐厅</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2024.03.17 19:30-03.17 21:00</t>
+          <t>2024.03.17 14:00-03.17 16:00</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="G17" t="n">
         <v>80</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80875</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81258</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/8AwIAy4I1705385447242.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/eysvN81k1705977896972.jpeg</t>
         </is>
       </c>
     </row>
@@ -2882,38 +2591,38 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2024-03-17</t>
+          <t>2024-03-21</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>上海·遇见新海诚--帝玖「这次一定」室内乐ACG音乐会</t>
+          <t>上海·春卷饭 十周年  2024  专场演出</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>延安东路523号 凯迪拉克·上海音乐厅</t>
+          <t>嘉兴路街道瑞虹路188号瑞虹天地月亮湾3层 Modern Sky LAB摩登天空(瑞虹天地店)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2024.03.17 14:00-03.17 16:00</t>
+          <t>2024.03.21 20:00-03.21 22:00</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>17</v>
+        <v>574</v>
       </c>
       <c r="G18" t="n">
-        <v>80</v>
+        <v>580</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81258</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81190</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/eysvN81k1705977896972.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/ho9rIMg21705894649801.jpeg</t>
         </is>
       </c>
     </row>
@@ -2923,38 +2632,38 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2024-03-21</t>
+          <t>2024-03-23</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>上海·春卷饭 十周年  2024  专场演出</t>
+          <t>上海·《卡农Canon in D》世界经典作品视听音乐会</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>嘉兴路街道瑞虹路188号瑞虹天地月亮湾3层 Modern Sky LAB摩登天空(瑞虹天地店)</t>
+          <t>南京西路1376号 上海商城剧院</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2024.03.21 20:00-03.21 22:00</t>
+          <t>2024.03.23 19:30-03.23 21:00</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>475</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>480</v>
+        <v>50</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81190</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81358</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/ho9rIMg21705894649801.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/Ctne29Xn1706089385959.png</t>
         </is>
       </c>
     </row>
@@ -2969,7 +2678,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>上海·《卡农Canon in D》世界经典作品视听音乐会</t>
+          <t>上海·《四月是你的谎言》友人A经典动漫音乐会</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2979,23 +2688,23 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2024.03.23 19:30-03.23 21:00</t>
+          <t>2024.03.23 15:00-03.23 16:30</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="G20" t="n">
         <v>50</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81358</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81361</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/Ctne29Xn1706089385959.png</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/wL0ZWVYi1706091574963.png</t>
         </is>
       </c>
     </row>
@@ -3005,38 +2714,38 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2024-03-23</t>
+          <t>2024-03-30</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>上海·《四月是你的谎言》友人A经典动漫音乐会</t>
+          <t>上海· TRUE（唐沢美帆）上海动漫交响音乐会</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>南京西路1376号 上海商城剧院</t>
+          <t>丁香路425号 上海东方艺术中心</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2024.03.23 15:00-03.23 16:30</t>
+          <t>2024.03.30 19:30-03.30 21:00</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>12</v>
+        <v>191</v>
       </c>
       <c r="G21" t="n">
-        <v>50</v>
+        <v>480</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81361</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80906</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/wL0ZWVYi1706091574963.png</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/FaJbLvS51705401178235.jpeg</t>
         </is>
       </c>
     </row>
@@ -3046,38 +2755,38 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2024-03-30</t>
+          <t>2024-04-06</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>上海· TRUE（唐沢美帆）上海动漫交响音乐会</t>
+          <t>上海·从Butter-Fly到夏目之爱してる —— “好想大声说爱你”动漫钢琴演奏会</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>丁香路425号 上海东方艺术中心</t>
+          <t>复兴中路1380号 捷豹上海交响音乐厅</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2024.03.30 19:30-03.30 21:00</t>
+          <t>2024.04.06 19:30-04.06 21:30</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>190</v>
+        <v>10</v>
       </c>
       <c r="G22" t="n">
-        <v>480</v>
+        <v>80</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80906</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80050</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/FaJbLvS51705401178235.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202312/0iJP3TY61703056498448.jpeg</t>
         </is>
       </c>
     </row>
@@ -3087,38 +2796,38 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2024-04-06</t>
+          <t>2024-04-13</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>上海·从Butter-Fly到夏目之爱してる —— “好想大声说爱你”动漫钢琴演奏会</t>
+          <t>上海·《四月是你的谎言》——“公生”与“薰”的钢琴小提琴唯美经典音乐集</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>复兴中路1380号 捷豹上海交响音乐厅</t>
+          <t>丁香路425号 上海东方艺术中心</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2024.04.06 19:30-04.06 21:30</t>
+          <t>2024.04.13 19:30-04.13 21:30</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>10</v>
+        <v>179</v>
       </c>
       <c r="G23" t="n">
         <v>80</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80050</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=78667</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202312/0iJP3TY61703056498448.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202311/bTP7w6GD1700130122940.jpeg</t>
         </is>
       </c>
     </row>
@@ -3128,38 +2837,38 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2024-04-13</t>
+          <t>2024-04-20</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>上海·《四月是你的谎言》——“公生”与“薰”的钢琴小提琴唯美经典音乐集</t>
+          <t>上海·Laurent Coulondre“心动巴黎”2024中国巡回音乐会</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>丁香路425号 上海东方艺术中心</t>
+          <t>汾阳路20号上海音乐学院内 上海贺绿汀音乐厅</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2024.04.13 19:30-04.13 21:30</t>
+          <t>2024.04.20 19:30-04.20 21:30</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>178</v>
+        <v>3</v>
       </c>
       <c r="G24" t="n">
         <v>80</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=78667</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81135</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202311/bTP7w6GD1700130122940.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/wXDdS5ap1705651730828.jpeg</t>
         </is>
       </c>
     </row>
@@ -3169,38 +2878,38 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2024-04-20</t>
+          <t>2024-04-26</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>上海·Laurent Coulondre“心动巴黎”2024中国巡回音乐会</t>
+          <t>上海· 夏川里美 2024 巡回演唱会 出道 25 周年纪念专场</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>汾阳路20号上海音乐学院内 上海贺绿汀音乐厅</t>
+          <t>东大名路889号 友邦大剧院</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2024.04.20 19:30-04.20 21:30</t>
+          <t>2024.04.26 19:30-04.26 21:30</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="G25" t="n">
-        <v>80</v>
+        <v>280</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81135</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81139</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/wXDdS5ap1705651730828.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/0Fj4cYOH1705652393930.jpeg</t>
         </is>
       </c>
     </row>
@@ -3210,77 +2919,36 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2024-04-26</t>
+          <t>2024-06-08</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>上海· 夏川里美 2024 巡回演唱会 出道 25 周年纪念专场</t>
+          <t>上海·菊次郎的夏天——久石让钢琴曲梦幻之旅演奏会</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>东大名路889号 友邦大剧院</t>
+          <t>延安东路523号 凯迪拉克·上海音乐厅</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2024.04.26 19:30-04.26 21:30</t>
+          <t>2024.06.08 19:30-06.08 21:00</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="G26" t="n">
-        <v>280</v>
+        <v>80</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81139</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81413</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
-        <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/0Fj4cYOH1705652393930.jpeg</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="1" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>2024-06-08</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>上海·菊次郎的夏天——久石让钢琴曲梦幻之旅演奏会</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>延安东路523号 凯迪拉克·上海音乐厅</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>2024.06.08 19:30-06.08 21:00</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>2</v>
-      </c>
-      <c r="G27" t="n">
-        <v>80</v>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81413</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
         <is>
           <t>//i2.hdslb.com/bfs/openplatform/202401/QqKuy4611706169245363.jpeg</t>
         </is>
@@ -3370,7 +3038,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="G2" t="n">
         <v>60</v>
@@ -3493,7 +3161,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2026</v>
+        <v>2030</v>
       </c>
       <c r="G5" t="n">
         <v>30</v>
@@ -3534,7 +3202,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2180</v>
+        <v>2197</v>
       </c>
       <c r="G6" t="n">
         <v>30</v>
@@ -3575,7 +3243,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="G7" t="n">
         <v>30</v>
@@ -3616,7 +3284,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>834</v>
+        <v>848</v>
       </c>
       <c r="G8" t="n">
         <v>10</v>
@@ -3739,7 +3407,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>948</v>
+        <v>990</v>
       </c>
       <c r="G11" t="n">
         <v>30</v>
@@ -3780,7 +3448,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="G12" t="n">
         <v>30</v>
@@ -3821,7 +3489,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="G13" t="n">
         <v>30</v>
@@ -3921,7 +3589,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="G2" t="n">
         <v>60</v>
@@ -3962,7 +3630,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>2026</v>
+        <v>2030</v>
       </c>
       <c r="G3" t="n">
         <v>30</v>
@@ -4003,7 +3671,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>2180</v>
+        <v>2197</v>
       </c>
       <c r="G4" t="n">
         <v>30</v>
@@ -4085,7 +3753,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1694</v>
+        <v>1696</v>
       </c>
       <c r="G6" t="n">
         <v>55</v>
@@ -4148,38 +3816,38 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2023-12-31</t>
+          <t>2023-12-27</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>上海·次元波板糖×时光代理人「锦瑟华年主题快闪店」</t>
+          <t>上海·爱乐汇《天空之城》久石让&amp;宫崎骏动漫经典音乐作品演奏会</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>西藏北路166静安大悦城北座6楼611号 次元波板糖</t>
+          <t>南京西路1376号 上海商城剧院</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2023.12.31 00:00-2024.01.29 23:59</t>
+          <t>2023.12.27 19:30-2024.02.03 12:00</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>858</v>
+        <v>51</v>
       </c>
       <c r="G8" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79972</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80103</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202312/z7bFCMqM1702972063289.png</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202312/2h2tIq7l1703144874867.png</t>
         </is>
       </c>
     </row>
@@ -4189,38 +3857,38 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2024-01-06</t>
+          <t>2023-12-31</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>上海·罗小黑 x HAPPY ZOO主题Cafe</t>
+          <t>上海·次元波板糖×时光代理人「锦瑟华年主题快闪店」</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>南京东路340号 百联zx创趣场</t>
+          <t>西藏北路166静安大悦城北座6楼611号 次元波板糖</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2024.01.06 00:00-02.29 23:59</t>
+          <t>2023.12.31 00:00-2024.01.29 23:59</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>834</v>
+        <v>859</v>
       </c>
       <c r="G9" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80171</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=79972</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202312/chPePM8d1703485388734.png</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202312/z7bFCMqM1702972063289.png</t>
         </is>
       </c>
     </row>
@@ -4230,38 +3898,38 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2024-01-22</t>
+          <t>2024-01-06</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>上海·「新春特惠」世嘉都市乐园-JP国潮杂技嘉年华</t>
+          <t>上海·罗小黑 x HAPPY ZOO主题Cafe</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>中山北路3300号环球港购物中心4楼 上海世嘉都市乐园</t>
+          <t>南京东路340号 百联zx创趣场</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2024.01.22 14:00-03.03 18:40</t>
+          <t>2024.01.06 00:00-02.29 23:59</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>848</v>
       </c>
       <c r="G10" t="n">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81210</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80171</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/sw2khwYM1706086166106.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202312/chPePM8d1703485388734.png</t>
         </is>
       </c>
     </row>
@@ -4271,38 +3939,38 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2024-01-27</t>
+          <t>2024-01-22</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>上海·同好召集令火影only</t>
+          <t>上海·「新春特惠」世嘉都市乐园-JP国潮杂技嘉年华</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>市真南路1199弄1号 智创TOP综合体产城</t>
+          <t>中山北路3300号环球港购物中心4楼 上海世嘉都市乐园</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2024.01.27 10:00-01.28 18:00</t>
+          <t>2024.01.22 14:00-03.03 18:40</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>575</v>
+        <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>88</v>
+        <v>49</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80284</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81210</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/9xGb6MXN1704183627126.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/sw2khwYM1706086166106.jpeg</t>
         </is>
       </c>
     </row>
@@ -4331,7 +3999,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1237</v>
+        <v>1239</v>
       </c>
       <c r="G12" t="n">
         <v>98</v>
@@ -4358,33 +4026,33 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>上海·魔都寒假漫展-CF01</t>
+          <t>上海・明日方舟主题店·[SWEET ZONE甜蜜区域]</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
+          <t>南京东路830号第一百货商业中心B馆5楼(海底捞旁边) 第一百货商业中心</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2024.01.27 10:00-01.28 16:00</t>
+          <t>2024.01.27 00:00-03.31 23:59</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1020</v>
+        <v>990</v>
       </c>
       <c r="G13" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80204</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81277</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202312/eK96fdcg1703573110264.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/hp6D0Drt1705991831205.jpeg</t>
         </is>
       </c>
     </row>
@@ -4394,38 +4062,38 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2024-01-27</t>
+          <t>2024-01-31</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>上海・明日方舟主题店·[SWEET ZONE甜蜜区域]</t>
+          <t>上海·寻迹冬日LOVELIVE同好会</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>南京东路830号第一百货商业中心B馆5楼(海底捞旁边) 第一百货商业中心</t>
+          <t>愚园路1250号 新歌空间</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2024.01.27 00:00-03.31 23:59</t>
+          <t>2024.01.31 11:30-01.31 17:00</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>948</v>
+        <v>194</v>
       </c>
       <c r="G14" t="n">
-        <v>30</v>
+        <v>83</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81277</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=79332</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/hp6D0Drt1705991831205.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202312/Ewreg1JT1701677993728.jpeg</t>
         </is>
       </c>
     </row>
@@ -4435,38 +4103,38 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2024-01-28</t>
+          <t>2024-02-01</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>上海 ·WOW潮元原神x星铁主题二次元狂欢派对</t>
+          <t>上海·次元波板糖×线条小狗MALTESE 主题快闪店</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>政通路189号五角场万达广场C栋 元气森林livehouse</t>
+          <t>西藏北路166静安大悦城北座6楼611号 次元波板糖</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2024.01.28 14:00-01.28 19:00</t>
+          <t>2024.02.01 00:00-03.01 23:59</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>456</v>
+        <v>179</v>
       </c>
       <c r="G15" t="n">
-        <v>149</v>
+        <v>30</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80167</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81345</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/QTp32HEM1705028548091.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/Qbpful951706080847394.png</t>
         </is>
       </c>
     </row>
@@ -4476,38 +4144,38 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2024-01-28</t>
+          <t>2024-02-02</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>上海·坏孩纸物语の第32届动漫节之冬日季</t>
+          <t>上海·2024《永远的7日之都》x  萌果酱谷子咖啡</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>剑川路1000号 闵行龙湖天街</t>
+          <t>南京东路340号百联ZX 萌果酱谷子咖啡（百联）</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2024.01.28 14:00-01.28 20:00</t>
+          <t>2024.02.02 00:00-03.10 23:59</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>746</v>
+        <v>42</v>
       </c>
       <c r="G16" t="n">
-        <v>36.9</v>
+        <v>30</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80871</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81357</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/5fmQrQJ81705573963752.png</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/5OYoWSGL1706087914805.jpeg</t>
         </is>
       </c>
     </row>
@@ -4517,38 +4185,38 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2024-01-28</t>
+          <t>2024-02-02</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>上海·次元裂缝-X 新年二次元偶像日</t>
+          <t>上海·次元LAB 二次元电音节</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>海潮路133号B1 JUMP工坊</t>
+          <t>中兴路1683号金融街购物中心L3-27 蜚声上海Livehouse</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2024.01.28 14:00-01.28 18:00</t>
+          <t>2024.02.02 12:30-02.02 21:00</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>90</v>
+        <v>682</v>
       </c>
       <c r="G17" t="n">
-        <v>70</v>
+        <v>380</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80999</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80128</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/lNroHqJY1705549448993.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202312/DEW1XYty1703226993965.jpeg</t>
         </is>
       </c>
     </row>
@@ -4558,38 +4226,38 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2024-01-31</t>
+          <t>2024-02-03</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>上海·寻迹冬日LOVELIVE同好会</t>
+          <t>上海·Coser迎春动漫展</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>愚园路1250号 新歌空间</t>
+          <t>海潮路133号B1 JUMP工坊</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2024.01.31 11:30-01.31 17:00</t>
+          <t>2024.02.03 10:00-02.04 17:00</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>194</v>
+        <v>912</v>
       </c>
       <c r="G18" t="n">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79332</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80646</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202312/Ewreg1JT1701677993728.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/4WVkFc4d1704787729064.jpeg</t>
         </is>
       </c>
     </row>
@@ -4599,38 +4267,38 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2024-02-01</t>
+          <t>2024-02-03</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>上海·次元波板糖×线条小狗MALTESE 主题快闪店</t>
+          <t>上海·ENP电次元派对vol.04</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>西藏北路166静安大悦城北座6楼611号 次元波板糖</t>
+          <t>人民大道221号 迪美购物中心</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2024.02.01 00:00-03.01 23:59</t>
+          <t>2024.02.03 18:30-02.03 22:00</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>167</v>
+        <v>24</v>
       </c>
       <c r="G19" t="n">
-        <v>30</v>
+        <v>99</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81345</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80945</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/Qbpful951706080847394.png</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/1sjalWS51705479361512.jpeg</t>
         </is>
       </c>
     </row>
@@ -4640,38 +4308,38 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2024-02-02</t>
+          <t>2024-02-03</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>上海·2024《永远的7日之都》x  萌果酱谷子咖啡</t>
+          <t>上海·偶像梦幻祭红白歌合战Only</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>南京东路340号百联ZX 萌果酱谷子咖啡（百联）</t>
+          <t>虹许路731号4号楼 THE BOXX•城市乐园</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2024.02.02 00:00-03.10 23:59</t>
+          <t>2024.02.03 13:30-02.03 22:00</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>35</v>
+        <v>105</v>
       </c>
       <c r="G20" t="n">
-        <v>30</v>
+        <v>88</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81357</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81199</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/5OYoWSGL1706087914805.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/C7E7svbZ1705903245860.jpeg</t>
         </is>
       </c>
     </row>
@@ -4681,38 +4349,38 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2024-02-02</t>
+          <t>2024-02-03</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>上海·次元LAB 二次元电音节</t>
+          <t>上海·第七届次元鹿角二次元派对</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>中兴路1683号金融街购物中心L3-27 蜚声上海Livehouse</t>
+          <t>长宁路1191号来福士西区(W)B1层01号、11号 星零界</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2024.02.02 12:30-02.02 21:00</t>
+          <t>2024.02.03 10:00-02.04 17:00</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>673</v>
+        <v>1346</v>
       </c>
       <c r="G21" t="n">
-        <v>380</v>
+        <v>98</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80128</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=79938</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202312/DEW1XYty1703226993965.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/b1XT2w4T1705027781100.jpeg</t>
         </is>
       </c>
     </row>
@@ -4722,38 +4390,38 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2024-02-03</t>
+          <t>2024-02-04</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>上海·Coser迎春动漫展</t>
+          <t>上海·触手猴钢琴巡演·marasy piano live tour『生音』上海站·Powered by 东方弹幕神乐失落幻想</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>海潮路133号B1 JUMP工坊</t>
+          <t>丁香路425号(上海科技馆地铁站1号口步行460米) 上海东方艺术中心音乐厅</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2024.02.03 10:00-02.04 17:00</t>
+          <t>2024.02.04 19:30-02.04 21:00</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>858</v>
+        <v>516</v>
       </c>
       <c r="G22" t="n">
-        <v>60</v>
+        <v>280</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80646</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80734</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/4WVkFc4d1704787729064.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/IcjPp0TE1704951328918.jpeg</t>
         </is>
       </c>
     </row>
@@ -4763,38 +4431,38 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2024-02-03</t>
+          <t>2024-02-10</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>上海·ENP电次元派对vol.04</t>
+          <t>上海·寒假CF漫展-春节档-神龙在世</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>人民大道221号 迪美购物中心</t>
+          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2024.02.03 18:30-02.03 22:00</t>
+          <t>2024.02.10 10:00-02.17 16:00</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="G23" t="n">
-        <v>99</v>
+        <v>49</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80945</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81192</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/1sjalWS51705479361512.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/S8XxkA631705896741998.jpeg</t>
         </is>
       </c>
     </row>
@@ -4804,38 +4472,38 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2024-02-03</t>
+          <t>2024-02-14</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>上海·偶像梦幻祭红白歌合战Only</t>
+          <t>上海·原X铁X崩only</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>虹许路731号4号楼 THE BOXX•城市乐园</t>
+          <t>澳门路168号 月星国际家居</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2024.02.03 13:30-02.03 22:00</t>
+          <t>2024.02.14 10:30-02.14 16:30</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>93</v>
+        <v>43</v>
       </c>
       <c r="G24" t="n">
-        <v>88</v>
+        <v>60</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81199</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81446</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/C7E7svbZ1705903245860.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/IIePRulM1706248855263.jpeg</t>
         </is>
       </c>
     </row>
@@ -4845,38 +4513,38 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2024-02-03</t>
+          <t>2024-02-14</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>上海·第七届次元鹿角二次元派对</t>
+          <t>上海·奇卡波利动漫嘉年华</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>长宁路1191号来福士西区(W)B1层01号、11号 星零界</t>
+          <t>申滨路36号 虹桥丽宝广场</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2024.02.03 10:00-02.04 17:00</t>
+          <t>2024.02.14 10:00-02.14 17:00</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>1331</v>
+        <v>77</v>
       </c>
       <c r="G25" t="n">
-        <v>98</v>
+        <v>48.8</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79938</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81260</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/b1XT2w4T1705027781100.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/9OHovK2V1705978109130.jpeg</t>
         </is>
       </c>
     </row>
@@ -4886,38 +4554,38 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2024-02-04</t>
+          <t>2024-02-14</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>上海·触手猴钢琴巡演·marasy piano live tour『生音』上海站·Powered by 东方弹幕神乐失落幻想</t>
+          <t>上海·魔都COS漫展-情人节专场AM01</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>丁香路425号(上海科技馆地铁站1号口步行460米) 上海东方艺术中心音乐厅</t>
+          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2024.02.04 19:30-02.04 21:00</t>
+          <t>2024.02.14 10:00-02.14 16:00</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>475</v>
+        <v>106</v>
       </c>
       <c r="G26" t="n">
-        <v>280</v>
+        <v>49</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80734</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80691</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/IcjPp0TE1704951328918.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/aSdjV6Kw1704868345679.jpeg</t>
         </is>
       </c>
     </row>
@@ -4927,38 +4595,38 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2024-02-10</t>
+          <t>2024-02-16</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>上海·寒假CF漫展-春节档-神龙在世</t>
+          <t>上海·次元裂缝-X 新年anikura派对</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
+          <t>海潮路133号B1 JUMP工坊</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2024.02.10 10:00-02.17 16:00</t>
+          <t>2024.02.16 14:00-02.16 19:00</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G27" t="n">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81192</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81314</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/S8XxkA631705896741998.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/OrhHWKdR1706062360956.jpeg</t>
         </is>
       </c>
     </row>
@@ -4968,38 +4636,38 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2024-02-14</t>
+          <t>2024-02-16</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>上海·原X铁X崩only</t>
+          <t>上海·第九届次元鹿角动漫游戏展</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>澳门路168号 月星国际家居</t>
+          <t>盈浦街道淀山浦社区淀山湖大道851号青浦万达茂F3 万达汽车乐园(青浦万达茂店)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2024.02.14 10:30-02.14 16:30</t>
+          <t>2024.02.16 11:00-02.17 18:00</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>28</v>
+        <v>1264</v>
       </c>
       <c r="G28" t="n">
-        <v>60</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81446</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80497</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/IIePRulM1706248855263.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/0duSXTQy1704423309244.jpeg</t>
         </is>
       </c>
     </row>
@@ -5009,38 +4677,38 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2024-02-14</t>
+          <t>2024-02-17</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>上海·奇卡波利动漫嘉年华</t>
+          <t>上海·少女番only2.0</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>申滨路36号 虹桥丽宝广场</t>
+          <t>营口路699号(黄兴公园地铁站2号口旁) 花嫁丽舍</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2024.02.14 10:00-02.14 17:00</t>
+          <t>2024.02.17 10:00-02.17 17:00</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>67</v>
+        <v>364</v>
       </c>
       <c r="G29" t="n">
-        <v>48.8</v>
+        <v>80</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81260</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81148</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/9OHovK2V1705978109130.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/j6eEZ18S1705657346664.jpeg</t>
         </is>
       </c>
     </row>
@@ -5050,38 +4718,38 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2024-02-14</t>
+          <t>2024-02-24</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>上海·魔都COS漫展-情人节专场AM01</t>
+          <t>上海·SISPmini动漫游戏嘉年华</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
+          <t>剑川路1000号 龙湖上海闵行天街</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2024.02.14 10:00-02.14 16:00</t>
+          <t>2024.02.24 13:00-02.25 19:00</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>101</v>
+        <v>434</v>
       </c>
       <c r="G30" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80691</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=79046</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/aSdjV6Kw1704868345679.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/jzovdppq1706166165502.jpeg</t>
         </is>
       </c>
     </row>
@@ -5091,38 +4759,38 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2024-02-16</t>
+          <t>2024-02-24</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>上海·次元裂缝-X 新年anikura派对</t>
+          <t>上海·原神×崩坏×星铁only旅行盛宴2.0</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>海潮路133号B1 JUMP工坊</t>
+          <t>西藏南路1号 上海大世界</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2024.02.16 14:00-02.16 19:00</t>
+          <t>2024.02.24 10:00-02.25 17:00</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>31</v>
+        <v>133</v>
       </c>
       <c r="G31" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81314</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81276</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/OrhHWKdR1706062360956.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/82hU3z8m1706155835021.png</t>
         </is>
       </c>
     </row>
@@ -5132,12 +4800,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2024-02-16</t>
+          <t>2024-02-24</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>上海·第九届次元鹿角动漫游戏展</t>
+          <t>上海·第三届燃梦BACG PRO游戏动漫展-原X铁X崩同好交流</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -5147,23 +4815,23 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2024.02.16 11:00-02.17 18:00</t>
+          <t>2024.02.24 11:00-02.25 16:30</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>1251</v>
+        <v>2514</v>
       </c>
       <c r="G32" t="n">
-        <v>65.90000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80497</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=77754</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/0duSXTQy1704423309244.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202312/7eGZETK91701943985671.jpeg</t>
         </is>
       </c>
     </row>
@@ -5173,38 +4841,38 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2024-02-17</t>
+          <t>2024-02-24</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>上海·少女番only2.0</t>
+          <t>上海·趣元界&amp;斗罗大陆上元佳节次元派对</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>营口路699号(黄兴公园地铁站2号口旁) 花嫁丽舍</t>
+          <t>长宁路1191号长宁来福士B1 长宁来福士</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2024.02.17 10:00-02.17 17:00</t>
+          <t>2024.02.24 11:30-02.25 17:30</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>351</v>
+        <v>511</v>
       </c>
       <c r="G33" t="n">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81148</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81415</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/j6eEZ18S1705657346664.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/yis4JHfE1706169986733.jpeg</t>
         </is>
       </c>
     </row>
@@ -5219,33 +4887,33 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>上海·SISPmini动漫游戏嘉年华</t>
+          <t>上海·魔都元宵节漫展-COS为王</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>剑川路1000号 龙湖上海闵行天街</t>
+          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2024.02.24 13:00-02.25 19:00</t>
+          <t>2024.02.24 10:00-02.25 16:00</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>426</v>
+        <v>11</v>
       </c>
       <c r="G34" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=79046</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81238</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/jzovdppq1706166165502.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/KxQZPADR1705913896609.jpeg</t>
         </is>
       </c>
     </row>
@@ -5260,33 +4928,33 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>上海·原神×崩坏×星铁only旅行盛宴2.0</t>
+          <t>上海·魔都多厨狂喜漫展-CH01</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>西藏南路1号 上海大世界</t>
+          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2024.02.24 10:00-02.25 17:00</t>
+          <t>2024.02.24 10:00-02.25 16:00</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>119</v>
+        <v>3</v>
       </c>
       <c r="G35" t="n">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81276</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81423</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/82hU3z8m1706155835021.png</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/axpOY3zo1706173660010.jpeg</t>
         </is>
       </c>
     </row>
@@ -5296,38 +4964,38 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2024-02-24</t>
+          <t>2024-03-02</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>上海·第三届燃梦BACG PRO游戏动漫展-原X铁X崩同好交流</t>
+          <t>上海·原神X星穹铁道ONLY</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>盈浦街道淀山浦社区淀山湖大道851号青浦万达茂F3 万达汽车乐园(青浦万达茂店)</t>
+          <t>逸仙路301号靠纪念路路口 上海宝丰联大酒店</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2024.02.24 11:00-02.25 16:30</t>
+          <t>2024.03.02 10:00-03.02 17:00</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2511</v>
+        <v>264</v>
       </c>
       <c r="G36" t="n">
-        <v>65.8</v>
+        <v>60</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=77754</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80299</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202312/7eGZETK91701943985671.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202312/V0xu26Cl1703753850690.jpeg</t>
         </is>
       </c>
     </row>
@@ -5337,38 +5005,38 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2024-02-24</t>
+          <t>2024-03-02</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>上海·趣元界&amp;斗罗大陆上元佳节次元派对</t>
+          <t>上海·小山百代2024上海粉丝见面会</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>长宁路1191号长宁来福士B1 长宁来福士</t>
+          <t>宜昌路179号 万代南梦宫上海文化中心</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2024.02.24 11:30-02.25 17:30</t>
+          <t>2024.03.02 13:00-03.02 20:00</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>509</v>
+        <v>253</v>
       </c>
       <c r="G37" t="n">
-        <v>98</v>
+        <v>380</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81415</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80924</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/yis4JHfE1706169986733.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/FpA9OkKy1705467080070.jpeg</t>
         </is>
       </c>
     </row>
@@ -5378,38 +5046,38 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2024-02-24</t>
+          <t>2024-03-03</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>上海·魔都元宵节漫展-COS为王</t>
+          <t>上海·怀旧番ONLY</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
+          <t>逸仙路270号  上海宝丰联大酒店</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2024.02.24 10:00-02.25 16:00</t>
+          <t>2024.03.03 10:00-03.03 17:00</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>11</v>
+        <v>155</v>
       </c>
       <c r="G38" t="n">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81238</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80575</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/KxQZPADR1705913896609.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/y4uWdyPT1704700763902.jpeg</t>
         </is>
       </c>
     </row>
@@ -5419,38 +5087,38 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2024-02-24</t>
+          <t>2024-03-09</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>上海·魔都多厨狂喜漫展-CH01</t>
+          <t>上海·S·CGE动漫游戏嘉年华</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>澳门路168号月星家居(江宁路地铁站1号口步行420米) 月星广场</t>
+          <t>军工路1076号 纪希片场(秀场)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2024.02.24 10:00-02.25 16:00</t>
+          <t>2024.03.09 10:00-03.10 17:00</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>1</v>
+        <v>73</v>
       </c>
       <c r="G39" t="n">
-        <v>49</v>
+        <v>70</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81423</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81173</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/axpOY3zo1706173660010.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/TYA5FLkE1705891815532.jpeg</t>
         </is>
       </c>
     </row>
@@ -5460,38 +5128,38 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2024-03-02</t>
+          <t>2024-03-09</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>上海·原神X星穹铁道ONLY</t>
+          <t>上海·爱乐之城音乐会</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>逸仙路301号靠纪念路路口 上海宝丰联大酒店</t>
+          <t>南京西路1376号 上海商城剧院</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2024.03.02 10:00-03.02 17:00</t>
+          <t>2024.03.09 14:00-03.09 15:30</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>260</v>
+        <v>2</v>
       </c>
       <c r="G40" t="n">
         <v>60</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80299</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81289</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202312/V0xu26Cl1703753850690.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/ZZXtDrwZ1705996679699.jpeg</t>
         </is>
       </c>
     </row>
@@ -5501,38 +5169,38 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2024-03-02</t>
+          <t>2024-03-09</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>上海·小山百代2024上海粉丝见面会</t>
+          <t>上海·青山刚昌ONLY【名侦探柯南&amp;魔术快斗】</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>宜昌路179号 万代南梦宫上海文化中心</t>
+          <t>漕宝路1688号 诺宝中心酒店</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2024.03.02 13:00-03.02 20:00</t>
+          <t>2024.03.09 10:00-03.09 16:30</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>249</v>
+        <v>896</v>
       </c>
       <c r="G41" t="n">
-        <v>380</v>
+        <v>73</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80924</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=76410</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/FpA9OkKy1705467080070.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202309/fVXMrcHy1693971682397.jpeg</t>
         </is>
       </c>
     </row>
@@ -5542,38 +5210,38 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2024-03-03</t>
+          <t>2024-03-16</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>上海·怀旧番ONLY</t>
+          <t>上海·三月的幻想演唱会2024「飞越蓝色时刻」</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>逸仙路270号  上海宝丰联大酒店</t>
+          <t>宜昌路179号 万代南梦宫上海文化中心</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2024.03.03 10:00-03.03 17:00</t>
+          <t>2024.03.16 19:00-03.16 20:30</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>153</v>
+        <v>52</v>
       </c>
       <c r="G42" t="n">
-        <v>60</v>
+        <v>380</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=80575</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80811</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/y4uWdyPT1704700763902.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/TO6xpSqr1705289483473.png</t>
         </is>
       </c>
     </row>
@@ -5583,38 +5251,38 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2024-03-09</t>
+          <t>2024-03-16</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>上海·S·CGE动漫游戏嘉年华</t>
+          <t>上海·坏孩纸物语の第33届动漫节之庄子篇</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>军工路1076号 纪希片场(秀场)</t>
+          <t>中山北路3300号4楼L4001号 环球港上海世嘉都市乐园</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2024.03.09 10:00-03.10 17:00</t>
+          <t>2024.03.16 10:00-03.17 21:00</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="G43" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81173</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81138</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/TYA5FLkE1705891815532.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/jpr1lCt21705652306481.png</t>
         </is>
       </c>
     </row>
@@ -5624,38 +5292,38 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2024-03-09</t>
+          <t>2024-03-17</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>上海·爱乐之城音乐会</t>
+          <t>上海·遇见新海诚--帝玖「这次一定」室内乐ACG音乐会</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>南京西路1376号 上海商城剧院</t>
+          <t>延安东路523号 凯迪拉克·上海音乐厅</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2024.03.09 14:00-03.09 15:30</t>
+          <t>2024.03.17 14:00-03.17 16:00</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="G44" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81289</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81258</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202401/ZZXtDrwZ1705996679699.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202401/eysvN81k1705977896972.jpeg</t>
         </is>
       </c>
     </row>
@@ -5665,38 +5333,38 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2024-03-09</t>
+          <t>2024-03-23</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>上海·青山刚昌ONLY【名侦探柯南&amp;魔术快斗】</t>
+          <t>上海·《四月是你的谎言》友人A经典动漫音乐会</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>漕宝路1688号 诺宝中心酒店</t>
+          <t>南京西路1376号 上海商城剧院</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2024.03.09 10:00-03.09 16:30</t>
+          <t>2024.03.23 15:00-03.23 16:30</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>893</v>
+        <v>14</v>
       </c>
       <c r="G45" t="n">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=76410</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=81361</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202309/fVXMrcHy1693971682397.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/wL0ZWVYi1706091574963.png</t>
         </is>
       </c>
     </row>
@@ -5706,38 +5374,38 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2024-03-17</t>
+          <t>2024-03-30</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>上海·遇见新海诚--帝玖「这次一定」室内乐ACG音乐会</t>
+          <t>上海· TRUE（唐沢美帆）上海动漫交响音乐会</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>延安东路523号 凯迪拉克·上海音乐厅</t>
+          <t>丁香路425号 上海东方艺术中心</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2024.03.17 14:00-03.17 16:00</t>
+          <t>2024.03.30 19:30-03.30 21:00</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>17</v>
+        <v>191</v>
       </c>
       <c r="G46" t="n">
-        <v>80</v>
+        <v>480</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81258</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=80906</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202401/eysvN81k1705977896972.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202401/FaJbLvS51705401178235.jpeg</t>
         </is>
       </c>
     </row>
@@ -5747,38 +5415,38 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2024-03-23</t>
+          <t>2024-04-13</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>上海·《四月是你的谎言》友人A经典动漫音乐会</t>
+          <t>上海·《四月是你的谎言》——“公生”与“薰”的钢琴小提琴唯美经典音乐集</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>南京西路1376号 上海商城剧院</t>
+          <t>丁香路425号 上海东方艺术中心</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2024.03.23 15:00-03.23 16:30</t>
+          <t>2024.04.13 19:30-04.13 21:30</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>12</v>
+        <v>179</v>
       </c>
       <c r="G47" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=81361</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=78667</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202401/wL0ZWVYi1706091574963.png</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202311/bTP7w6GD1700130122940.jpeg</t>
         </is>
       </c>
     </row>
@@ -5788,38 +5456,38 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2024-04-13</t>
+          <t>2024-04-27</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>上海·《四月是你的谎言》——“公生”与“薰”的钢琴小提琴唯美经典音乐集</t>
+          <t>上海·  第五十三届妖漫动漫游戏展</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>丁香路425号 上海东方艺术中心</t>
+          <t>曹杨路1888号 复悦荟</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2024.04.13 19:30-04.13 21:30</t>
+          <t>2024.04.27 10:00-04.27 17:00</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>178</v>
+        <v>150</v>
       </c>
       <c r="G48" t="n">
         <v>80</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=78667</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=78657</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202311/bTP7w6GD1700130122940.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202401/tamNdgEN1705331335847.jpeg</t>
         </is>
       </c>
     </row>
@@ -5848,7 +5516,7 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G49" t="n">
         <v>70</v>
@@ -5889,7 +5557,7 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="G50" t="n">
         <v>79</v>

</xml_diff>